<commit_message>
feat(F-NAR-016): TREE-DIF-047 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-047.xlsx
+++ b/stories/arbres/TREE-DIF-047.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un grillon chante, tout bas, derrière le volet. Ça sent encore le savon, dans le couloir. La chambre de Nino garde une lampe ronde. Elle fait un cercle pâle, au plafond. Tes chaussettes sont trop chaudes, Nino ? Un peu, papa. Maman pose l'oreiller rayé sur le tapis. Il attend le camp, tu le vois ? Il veut dormir, tout grand. En ce moment, Nino touche la lampe torche. Je veux camper ici, toute la nuit. On prépare les affaires, alors ? La lampe, le sac, et l'oreiller. Merci, tu tiens la lampe tout droit.</t>
+          <t>Un grillon chante, tout bas, derrière le volet. Ça sent encore le savon, dans le couloir. L'abat-jour de Nino fait un cercle pâle. Le plafond garde une lune ronde, toute douce. Tes chaussettes sont trop chaudes, Nino ? Un peu, papa. Maman pose l'oreiller rayé sur le tapis. Il attend le camp, tu le vois ? Il veut dormir, tout grand. En ce moment, Nino touche la lampe torche. Je veux camper ici, toute la nuit. On prépare les affaires, alors ? La lampe, le sac, et l'oreiller. Merci, tu tiens la lampe tout droit.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un grillon chante, tout bas, derrière le volet. Ça sent encore le savon, dans le couloir. La chambre de Nino garde une lampe ronde. Elle fait un cercle pâle, au plafond. Tes chaussettes sont trop chaudes, Nino ? Un peu, papa. Maman pose l'oreiller rayé sur le tapis. Il attend le camp, tu le vois ? Il veut dormir, tout grand. En ce moment, Nino touche la lampe torche. Je veux camper ici, toute la nuit. On prépare les affaires, alors ? La lampe, le sac, et l'oreiller. Merci, tu tiens la lampe tout droit.</t>
+          <t>Un grillon chante, tout bas, derrière le volet. Ça sent encore le savon, dans le couloir. L'abat-jour de Nino fait un cercle pâle. Le plafond garde une lune ronde, toute douce. Tes chaussettes sont trop chaudes, Nino ? Un peu, papa. Maman pose l'oreiller rayé sur le tapis. Il attend le camp, tu le vois ? Il veut dormir, tout grand. En ce moment, Nino touche la lampe torche. Je veux camper ici, toute la nuit. On prépare les affaires, alors ? La lampe, le sac, et l'oreiller. Merci, tu tiens la lampe tout droit.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1339,8 +1339,8 @@
         <is>
           <t>narrateur|Un grillon chante, tout bas, derrière le volet.
 narrateur|Ça sent encore le savon, dans le couloir.
-narrateur|La chambre de Nino garde une lampe ronde.
-narrateur|Elle fait un cercle pâle, au plafond.
+narrateur|L'abat-jour de Nino fait un cercle pâle.
+narrateur|Le plafond garde une lune ronde, toute douce.
 papa|Tes chaussettes sont trop chaudes, Nino ?
 enfant-m|Un peu, papa.
 narrateur|Maman pose l'oreiller rayé sur le tapis.
@@ -1930,12 +1930,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Dans les mains. Oui. La lampe torche tient, déjà un peu chaude. C'est pour le camp, papa. Nino a les genoux plus hauts que d'habitude. Ses pieds n'arrêtent pas de bouger. Il a beaucoup d'élan, c'est tout. On reste dans la chambre ? Oui, papa.</t>
+          <t>Dans les mains. Oui. Un clic de lampe réveille le plafond. C'est mon soleil de camp. Nino plie un genou, puis l'autre, trop vite. Le faisceau dessine un lapin, puis le perd. Tes pieds veulent déjà la nuit. On pose le camp ici ? Oui, papa.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Dans les mains. Oui. La lampe torche tient, déjà un peu chaude. C'est pour le camp, papa. Nino a les genoux plus hauts que d'habitude. Ses pieds n'arrêtent pas de bouger. Il a beaucoup d'élan, c'est tout. On reste dans la chambre ? Oui, papa.</t>
+          <t>Dans les mains. Oui. Un clic de lampe réveille le plafond. C'est mon soleil de camp. Nino plie un genou, puis l'autre, trop vite. Le faisceau dessine un lapin, puis le perd. Tes pieds veulent déjà la nuit. On pose le camp ici ? Oui, papa.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2076,12 +2076,12 @@
         <is>
           <t>enfant-m|Dans les mains.
 maman|Oui.
-narrateur|La lampe torche tient, déjà un peu chaude.
-enfant-m|C'est pour le camp, papa.
-narrateur|Nino a les genoux plus hauts que d'habitude.
-narrateur|Ses pieds n'arrêtent pas de bouger.
-maman|Il a beaucoup d'élan, c'est tout.
-papa|On reste dans la chambre ?
+narrateur|Un clic de lampe réveille le plafond.
+enfant-m|C'est mon soleil de camp.
+narrateur|Nino plie un genou, puis l'autre, trop vite.
+narrateur|Le faisceau dessine un lapin, puis le perd.
+maman|Tes pieds veulent déjà la nuit.
+papa|On pose le camp ici ?
 enfant-m|Oui, papa.</t>
         </is>
       </c>
@@ -2109,12 +2109,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Nino tapote déjà le parquet, tout léger. La fenêtre garde un rai de rue. Le tapis fait un carré chaud. Le pied du lit attend, tout bas. On campe où, Nino ?</t>
+          <t>Nino tapote déjà le parquet, tout léger. Sous la fenêtre, le rideau garde un rai de rue. Au milieu, le tapis fait un carré chaud. Près du bois, le pied du lit attend. On campe où, Nino ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Nino tapote déjà le parquet, tout léger. La fenêtre garde un rai de rue. Le tapis fait un carré chaud. Le pied du lit attend, tout bas. On campe où, Nino ?</t>
+          <t>Nino tapote déjà le parquet, tout léger. Sous la fenêtre, le rideau garde un rai de rue. Au milieu, le tapis fait un carré chaud. Près du bois, le pied du lit attend. On campe où, Nino ?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2274,9 +2274,9 @@
       <c r="AW7" t="inlineStr">
         <is>
           <t>narrateur|Nino tapote déjà le parquet, tout léger.
-narrateur|La fenêtre garde un rai de rue.
-narrateur|Le tapis fait un carré chaud.
-narrateur|Le pied du lit attend, tout bas.
+narrateur|Sous la fenêtre, le rideau garde un rai de rue.
+narrateur|Au milieu, le tapis fait un carré chaud.
+narrateur|Près du bois, le pied du lit attend.
 papa|On campe où, Nino ?</t>
         </is>
       </c>
@@ -2304,12 +2304,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>La lampe torche voyage vers la fenêtre. Nino tape le parquet, trop vite. Moi je cours, papa ! Ses pieds font des ronds, trop larges. Le faisceau court sur le rideau, trop vite. La lampe torche n'attendait pas ça. Il a envie de bouger, c'est tout. Tes jambes sont plus vives, ce soir. On campe comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Nino porte la lampe vers le rideau. Ses talons tambourinent le parquet. Le camp, c'est là, papa ! Le faisceau devient un lapin, puis s'enfuit. La lampe torche part trop vite. Tes pieds dansent, ce soir. Le rideau n'est pas encore une tente. On campe comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>La lampe torche voyage vers la fenêtre. Nino tape le parquet, trop vite. Moi je cours, papa ! Ses pieds font des ronds, trop larges. Le faisceau court sur le rideau, trop vite. La lampe torche n'attendait pas ça. Il a envie de bouger, c'est tout. Tes jambes sont plus vives, ce soir. On campe comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Nino porte la lampe vers le rideau. Ses talons tambourinent le parquet. Le camp, c'est là, papa ! Le faisceau devient un lapin, puis s'enfuit. La lampe torche part trop vite. Tes pieds dansent, ce soir. Le rideau n'est pas encore une tente. On campe comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2444,14 +2444,13 @@
       <c r="AV8" s="2" t="inlineStr"/>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>narrateur|La lampe torche voyage vers la fenêtre.
-narrateur|Nino tape le parquet, trop vite.
-enfant-m|Moi je cours, papa !
-narrateur|Ses pieds font des ronds, trop larges.
-narrateur|Le faisceau court sur le rideau, trop vite.
-enfant-m|La lampe torche n'attendait pas ça.
-maman|Il a envie de bouger, c'est tout.
-papa|Tes jambes sont plus vives, ce soir.
+          <t>narrateur|Nino porte la lampe vers le rideau.
+narrateur|Ses talons tambourinent le parquet.
+enfant-m|Le camp, c'est là, papa !
+narrateur|Le faisceau devient un lapin, puis s'enfuit.
+enfant-m|La lampe torche part trop vite.
+maman|Tes pieds dansent, ce soir.
+papa|Le rideau n'est pas encore une tente.
 enfant-m|On campe comment, alors ?
 papa|Tu fais comment, avec nous ?</t>
         </is>
@@ -2480,12 +2479,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Nino tape encore le parquet, tout fort. Les lucioles, le rideau, ou maman ?</t>
+          <t>Le lapin de lumière court encore. Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Nino tape encore le parquet, tout fort. Les lucioles, le rideau, ou maman ?</t>
+          <t>Le lapin de lumière court encore. Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2644,7 +2643,7 @@
       <c r="AV9" s="2" t="inlineStr"/>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|Nino tape encore le parquet, tout fort.
+          <t>narrateur|Le lapin de lumière court encore.
 papa|Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
@@ -2672,12 +2671,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>On joue aux lucioles. Toi tu bouges, moi je suis le rond. Nino tient la lampe, le faisceau danse. Deux ronds se croisent sur le rideau. Nino saute une fois, puis s'arrête. Maintenant c'est le camp. L'élan a trouvé sa fenêtre. Vous jouez à tour, sur le tissu. Le rideau redevient un mur, tout doux.</t>
+          <t>On joue aux lucioles. Toi tu clignes, moi je compte. Nino cligne la lampe, un, deux, trois. Des points d'or s'allument sur le rideau. Nino cligne encore, puis s'arrête. Les lucioles sont fatiguées. Le camp a sa lumière, maintenant. Vous avez dansé, puis posé. Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>On joue aux lucioles. Toi tu bouges, moi je suis le rond. Nino tient la lampe, le faisceau danse. Deux ronds se croisent sur le rideau. Nino saute une fois, puis s'arrête. Maintenant c'est le camp. L'élan a trouvé sa fenêtre. Vous jouez à tour, sur le tissu. Le rideau redevient un mur, tout doux.</t>
+          <t>On joue aux lucioles. Toi tu clignes, moi je compte. Nino cligne la lampe, un, deux, trois. Des points d'or s'allument sur le rideau. Nino cligne encore, puis s'arrête. Les lucioles sont fatiguées. Le camp a sa lumière, maintenant. Vous avez dansé, puis posé. Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2813,14 +2812,14 @@
       <c r="AW10" t="inlineStr">
         <is>
           <t>enfant-m|On joue aux lucioles.
-papa|Toi tu bouges, moi je suis le rond.
-narrateur|Nino tient la lampe, le faisceau danse.
-narrateur|Deux ronds se croisent sur le rideau.
-narrateur|Nino saute une fois, puis s'arrête.
-enfant-m|Maintenant c'est le camp.
-maman|L'élan a trouvé sa fenêtre.
-papa|Vous jouez à tour, sur le tissu.
-narrateur|Le rideau redevient un mur, tout doux.</t>
+papa|Toi tu clignes, moi je compte.
+narrateur|Nino cligne la lampe, un, deux, trois.
+narrateur|Des points d'or s'allument sur le rideau.
+narrateur|Nino cligne encore, puis s'arrête.
+enfant-m|Les lucioles sont fatiguées.
+maman|Le camp a sa lumière, maintenant.
+papa|Vous avez dansé, puis posé.
+narrateur|Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
     </row>
@@ -2847,12 +2846,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le dernier rond du rideau est à eux. On a joué, chacun son tour. Toi tu bougais, moi je suivais. Vous avez laissé l'élan dessiner. La chambre sent encore le savon. La lampe torche garde un rond tiède, tout petit. Un trait clair dort sur le bois. On s'allonge, papa. Les chaussettes retrouvent le tapis tiède.</t>
+          <t>Nino s'allonge, le sac sous le rideau. Les lucioles sont couchées, papa. Toi tu clignais, moi je comptais. Le camp a sa lumière, ce soir. La chambre sent encore le savon. La lampe torche garde un rond tiède, tout petit. Un point d'or dort sur le tissu. Bonne nuit, fenêtre. Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Le dernier rond du rideau est à eux. On a joué, chacun son tour. Toi tu bougais, moi je suivais. Vous avez laissé l'élan dessiner. La chambre sent encore le savon. La lampe torche garde un rond tiède, tout petit. Un trait clair dort sur le bois. On s'allonge, papa. Les chaussettes retrouvent le tapis tiède.</t>
+          <t>Nino s'allonge, le sac sous le rideau. Les lucioles sont couchées, papa. Toi tu clignais, moi je comptais. Le camp a sa lumière, ce soir. La chambre sent encore le savon. La lampe torche garde un rond tiède, tout petit. Un point d'or dort sur le tissu. Bonne nuit, fenêtre. Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2987,14 +2986,14 @@
       <c r="AV11" s="2" t="inlineStr"/>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|Le dernier rond du rideau est à eux.
-enfant-m|On a joué, chacun son tour.
-papa|Toi tu bougais, moi je suivais.
-maman|Vous avez laissé l'élan dessiner.
+          <t>narrateur|Nino s'allonge, le sac sous le rideau.
+enfant-m|Les lucioles sont couchées, papa.
+papa|Toi tu clignais, moi je comptais.
+maman|Le camp a sa lumière, ce soir.
 narrateur|La chambre sent encore le savon.
 narrateur|La lampe torche garde un rond tiède, tout petit.
-narrateur|Un trait clair dort sur le bois.
-enfant-m|On s'allonge, papa.
+narrateur|Un point d'or dort sur le tissu.
+enfant-m|Bonne nuit, fenêtre.
 narrateur|Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
@@ -3022,12 +3021,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu. Nino pose les genoux au bois. La lampe torche attend près du rebord. Sa respiration redevient calme, tout doux. Je suis prêt ? Le rideau ne bouge plus. Vous avez laissé l'élan s'asseoir. Le faisceau tient enfin, tout droit. Le camp peut s'ouvrir.</t>
+          <t>On attend le rideau. Nino pose les genoux au parquet. La lampe repose contre le rebord, éteinte. Le volet tape une fois, puis plus. Il ne bouge plus ? Le tissu est calme, oui. Tes pieds se sont assis, eux aussi. Nino rallume, tout droit, tout petit. Le camp peut s'ouvrir.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu. Nino pose les genoux au bois. La lampe torche attend près du rebord. Sa respiration redevient calme, tout doux. Je suis prêt ? Le rideau ne bouge plus. Vous avez laissé l'élan s'asseoir. Le faisceau tient enfin, tout droit. Le camp peut s'ouvrir.</t>
+          <t>On attend le rideau. Nino pose les genoux au parquet. La lampe repose contre le rebord, éteinte. Le volet tape une fois, puis plus. Il ne bouge plus ? Le tissu est calme, oui. Tes pieds se sont assis, eux aussi. Nino rallume, tout droit, tout petit. Le camp peut s'ouvrir.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3162,14 +3161,14 @@
       <c r="AV12" s="2" t="inlineStr"/>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>enfant-m|On attend un peu.
-narrateur|Nino pose les genoux au bois.
-narrateur|La lampe torche attend près du rebord.
-narrateur|Sa respiration redevient calme, tout doux.
-enfant-m|Je suis prêt ?
-maman|Le rideau ne bouge plus.
-papa|Vous avez laissé l'élan s'asseoir.
-narrateur|Le faisceau tient enfin, tout droit.
+          <t>enfant-m|On attend le rideau.
+narrateur|Nino pose les genoux au parquet.
+narrateur|La lampe repose contre le rebord, éteinte.
+narrateur|Le volet tape une fois, puis plus.
+enfant-m|Il ne bouge plus ?
+maman|Le tissu est calme, oui.
+papa|Tes pieds se sont assis, eux aussi.
+narrateur|Nino rallume, tout droit, tout petit.
 enfant-m|Le camp peut s'ouvrir.</t>
         </is>
       </c>
@@ -3197,12 +3196,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Le rebord de la fenêtre garde encore la chaleur. Je me suis arrêté, d'abord. Puis le faisceau est resté droit. L'élan s'est assis, puis il a campé. Le rideau redevient calme. La lampe torche garde un rond tiède, tout petit. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
+          <t>Nino s'allonge, le rideau tout calme. J'ai attendu le volet, d'abord. Puis le faisceau est resté droit. Tes pieds se sont assis, eux aussi. Le tissu ne danse plus. La lampe torche garde un rond tiède, tout petit. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Le rebord de la fenêtre garde encore la chaleur. Je me suis arrêté, d'abord. Puis le faisceau est resté droit. L'élan s'est assis, puis il a campé. Le rideau redevient calme. La lampe torche garde un rond tiède, tout petit. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
+          <t>Nino s'allonge, le rideau tout calme. J'ai attendu le volet, d'abord. Puis le faisceau est resté droit. Tes pieds se sont assis, eux aussi. Le tissu ne danse plus. La lampe torche garde un rond tiède, tout petit. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3337,11 +3336,11 @@
       <c r="AV13" s="2" t="inlineStr"/>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|Le rebord de la fenêtre garde encore la chaleur.
-enfant-m|Je me suis arrêté, d'abord.
+          <t>narrateur|Nino s'allonge, le rideau tout calme.
+enfant-m|J'ai attendu le volet, d'abord.
 papa|Puis le faisceau est resté droit.
-maman|L'élan s'est assis, puis il a campé.
-narrateur|Le rideau redevient calme.
+maman|Tes pieds se sont assis, eux aussi.
+narrateur|Le tissu ne danse plus.
 narrateur|La lampe torche garde un rond tiède, tout petit.
 narrateur|Une poussière reste coincée, tout près.
 enfant-m|À demain, les ronds.
@@ -3372,12 +3371,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens la lampe ? Je la tiens, un pas chacun. Maman pose la lampe près de sa main. Nino pose un pied, puis l'autre. Le faisceau reste sage, juste à côté. On demande, et ça va ! Vous avez demandé, tout calme. Ma main a juste attendu. La fenêtre garde un rai, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu poses le camp. Maman prend la lampe, Nino tend le sac. Nino étale le sac sous le rai de rue. Le faisceau reste sage, dans sa main. Toi tu tiens, moi je range. Vous avez demandé, et ça tient. Ma main fait le piquet, ce soir. La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens la lampe ? Je la tiens, un pas chacun. Maman pose la lampe près de sa main. Nino pose un pied, puis l'autre. Le faisceau reste sage, juste à côté. On demande, et ça va ! Vous avez demandé, tout calme. Ma main a juste attendu. La fenêtre garde un rai, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu poses le camp. Maman prend la lampe, Nino tend le sac. Nino étale le sac sous le rai de rue. Le faisceau reste sage, dans sa main. Toi tu tiens, moi je range. Vous avez demandé, et ça tient. Ma main fait le piquet, ce soir. La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3512,14 +3511,14 @@
       <c r="AV14" s="2" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>enfant-m|Maman, tu tiens la lampe ?
-maman|Je la tiens, un pas chacun.
-narrateur|Maman pose la lampe près de sa main.
-narrateur|Nino pose un pied, puis l'autre.
-narrateur|Le faisceau reste sage, juste à côté.
-enfant-m|On demande, et ça va !
-papa|Vous avez demandé, tout calme.
-maman|Ma main a juste attendu.
+          <t>enfant-m|Maman, tu tiens, s'il te plaît ?
+maman|Je tiens, tu poses le camp.
+narrateur|Maman prend la lampe, Nino tend le sac.
+narrateur|Nino étale le sac sous le rai de rue.
+narrateur|Le faisceau reste sage, dans sa main.
+enfant-m|Toi tu tiens, moi je range.
+papa|Vous avez demandé, et ça tient.
+maman|Ma main fait le piquet, ce soir.
 narrateur|La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
@@ -3547,12 +3546,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>La main de maman reste dans l'air, tout légère. J'ai attendu le pas. On a demandé, et ça allait. Sa main a tenu vos pieds. La chambre vous rend le silence. La lampe torche pose un grain de lumière sur le bois. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
+          <t>Nino s'allonge, la main de maman tout près. Tu tenais le piquet. Vous avez demandé, et ça tenait. Ma main a fait la tente. La chambre rend le silence, tout doux. La lampe torche pose un grain de lumière. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>La main de maman reste dans l'air, tout légère. J'ai attendu le pas. On a demandé, et ça allait. Sa main a tenu vos pieds. La chambre vous rend le silence. La lampe torche pose un grain de lumière sur le bois. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
+          <t>Nino s'allonge, la main de maman tout près. Tu tenais le piquet. Vous avez demandé, et ça tenait. Ma main a fait la tente. La chambre rend le silence, tout doux. La lampe torche pose un grain de lumière. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3687,12 +3686,12 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|La main de maman reste dans l'air, tout légère.
-enfant-m|J'ai attendu le pas.
-papa|On a demandé, et ça allait.
-maman|Sa main a tenu vos pieds.
-narrateur|La chambre vous rend le silence.
-narrateur|La lampe torche pose un grain de lumière sur le bois.
+          <t>narrateur|Nino s'allonge, la main de maman tout près.
+enfant-m|Tu tenais le piquet.
+papa|Vous avez demandé, et ça tenait.
+maman|Ma main a fait la tente.
+narrateur|La chambre rend le silence, tout doux.
+narrateur|La lampe torche pose un grain de lumière.
 narrateur|Nino touche le rideau, du bout.
 enfant-m|Il est à nous.
 narrateur|Un rai de rue barre encore le tissu.</t>
@@ -3722,12 +3721,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>La lampe torche s'arrête au milieu du tapis. Le tapis est à nous, maman. Ses pieds quittent le tissu, puis reviennent. Les genoux de Nino chassent le faisceau, trop loin. Un peu de poussière lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, trop vite. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Nino pose la lampe au milieu du tapis. Ici, c'est la clairière, maman. Ses genoux font un petit trampoline. Le faisceau roule, et le rond se perd. Un fil de laine se lève, puis retombe. Ton corps veut encore courir. Le tapis n'a pas encore de tente. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>La lampe torche s'arrête au milieu du tapis. Le tapis est à nous, maman. Ses pieds quittent le tissu, puis reviennent. Les genoux de Nino chassent le faisceau, trop loin. Un peu de poussière lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, trop vite. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Nino pose la lampe au milieu du tapis. Ici, c'est la clairière, maman. Ses genoux font un petit trampoline. Le faisceau roule, et le rond se perd. Un fil de laine se lève, puis retombe. Ton corps veut encore courir. Le tapis n'a pas encore de tente. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3862,13 +3861,13 @@
       <c r="AV16" s="2" t="inlineStr"/>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>narrateur|La lampe torche s'arrête au milieu du tapis.
-enfant-m|Le tapis est à nous, maman.
-narrateur|Ses pieds quittent le tissu, puis reviennent.
-narrateur|Les genoux de Nino chassent le faisceau, trop loin.
-narrateur|Un peu de poussière lève, puis retombe.
-maman|Il a de l'élan, comme un petit vent.
-papa|Toi tu vas plus loin, trop vite.
+          <t>narrateur|Nino pose la lampe au milieu du tapis.
+enfant-m|Ici, c'est la clairière, maman.
+narrateur|Ses genoux font un petit trampoline.
+narrateur|Le faisceau roule, et le rond se perd.
+narrateur|Un fil de laine se lève, puis retombe.
+maman|Ton corps veut encore courir.
+papa|Le tapis n'a pas encore de tente.
 enfant-m|On peut jouer avec, quand même ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -3897,12 +3896,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore sur le tapis. Le sentier, la fermeture, ou papa ?</t>
+          <t>Le sac n'a pas encore de forme. Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore sur le tapis. Le sentier, la fermeture, ou papa ?</t>
+          <t>Le sac n'a pas encore de forme. Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -4061,7 +4060,7 @@
       <c r="AV17" s="2" t="inlineStr"/>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|Nino rebondit encore sur le tapis.
+          <t>narrateur|Le sac n'a pas encore de forme.
 maman|Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
@@ -4089,12 +4088,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On fait un sentier. Toi derrière, moi devant ! Nino garde la lampe, papa saute devant. Deux ombres passent sur le même tapis. Nino va plus vite, papa plus loin. On arrive au bout, tous les deux. Vous avez joué avec l'élan. Le tapis vous a laissés passer. Un fil de laine reste, tout petit.</t>
+          <t>On fait un sentier. Toi tu sautes, moi je suis derrière. Nino pose la lampe, papa marque le sentier. Des pas dessinent un chemin sur le tapis. Nino saute une case, papa une autre. La clairière est au bout. Vous avez joué, puis posé le sac. Le tapis est devenu un chemin. Un fil de laine reste, tout petit.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>On fait un sentier. Toi derrière, moi devant ! Nino garde la lampe, papa saute devant. Deux ombres passent sur le même tapis. Nino va plus vite, papa plus loin. On arrive au bout, tous les deux. Vous avez joué avec l'élan. Le tapis vous a laissés passer. Un fil de laine reste, tout petit.</t>
+          <t>On fait un sentier. Toi tu sautes, moi je suis derrière. Nino pose la lampe, papa marque le sentier. Des pas dessinent un chemin sur le tapis. Nino saute une case, papa une autre. La clairière est au bout. Vous avez joué, puis posé le sac. Le tapis est devenu un chemin. Un fil de laine reste, tout petit.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4230,13 +4229,13 @@
       <c r="AW18" t="inlineStr">
         <is>
           <t>enfant-m|On fait un sentier.
-papa|Toi derrière, moi devant !
-narrateur|Nino garde la lampe, papa saute devant.
-narrateur|Deux ombres passent sur le même tapis.
-narrateur|Nino va plus vite, papa plus loin.
-enfant-m|On arrive au bout, tous les deux.
-maman|Vous avez joué avec l'élan.
-papa|Le tapis vous a laissés passer.
+papa|Toi tu sautes, moi je suis derrière.
+narrateur|Nino pose la lampe, papa marque le sentier.
+narrateur|Des pas dessinent un chemin sur le tapis.
+narrateur|Nino saute une case, papa une autre.
+enfant-m|La clairière est au bout.
+maman|Vous avez joué, puis posé le sac.
+papa|Le tapis est devenu un chemin.
 narrateur|Un fil de laine reste, tout petit.</t>
         </is>
       </c>
@@ -4264,12 +4263,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Deux paires de chaussettes marquent le bout du tapis. Toi devant, moi derrière. Tes jambes allaient plus loin. Vous avez sauté avec l'élan, pas contre. Le tapis redevient chaud, et calme. La lampe torche garde un rond tiède, tout petit. Un peu de laine sèche déjà sur le tissu. On s'allonge, le sentier reste. Le lit fait une ombre longue.</t>
+          <t>Nino s'allonge au bout du sentier. Toi devant, moi derrière. Tes sauts ont fait le chemin. La clairière est devenue un camp. Le tapis redevient chaud, et calme. La lampe torche garde un rond tiède, tout petit. Un peu de laine sèche déjà. Le sentier reste, maman. Le lit fait une ombre longue.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Deux paires de chaussettes marquent le bout du tapis. Toi devant, moi derrière. Tes jambes allaient plus loin. Vous avez sauté avec l'élan, pas contre. Le tapis redevient chaud, et calme. La lampe torche garde un rond tiède, tout petit. Un peu de laine sèche déjà sur le tissu. On s'allonge, le sentier reste. Le lit fait une ombre longue.</t>
+          <t>Nino s'allonge au bout du sentier. Toi devant, moi derrière. Tes sauts ont fait le chemin. La clairière est devenue un camp. Le tapis redevient chaud, et calme. La lampe torche garde un rond tiède, tout petit. Un peu de laine sèche déjà. Le sentier reste, maman. Le lit fait une ombre longue.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4404,14 +4403,14 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|Deux paires de chaussettes marquent le bout du tapis.
+          <t>narrateur|Nino s'allonge au bout du sentier.
 enfant-m|Toi devant, moi derrière.
-papa|Tes jambes allaient plus loin.
-maman|Vous avez sauté avec l'élan, pas contre.
+papa|Tes sauts ont fait le chemin.
+maman|La clairière est devenue un camp.
 narrateur|Le tapis redevient chaud, et calme.
 narrateur|La lampe torche garde un rond tiède, tout petit.
-narrateur|Un peu de laine sèche déjà sur le tissu.
-enfant-m|On s'allonge, le sentier reste.
+narrateur|Un peu de laine sèche déjà.
+enfant-m|Le sentier reste, maman.
 narrateur|Le lit fait une ombre longue.</t>
         </is>
       </c>
@@ -4439,12 +4438,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient la lampe, sur le tissu. La fermeture avance, tout seule d'abord. Nino souffle, puis il recule. C'est à toi, Nino. Merci, j'y vais. Chacun son tour, sur le tapis. L'élan a attendu la place.</t>
+          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient la lampe, le sac attend. Le zip avance, dent après dent. Nino souffle, les épaules baissent. C'est à toi, Nino. J'y glisse un pied. Chacun son tour, sur le tapis. La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient la lampe, sur le tissu. La fermeture avance, tout seule d'abord. Nino souffle, puis il recule. C'est à toi, Nino. Merci, j'y vais. Chacun son tour, sur le tapis. L'élan a attendu la place.</t>
+          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient la lampe, le sac attend. Le zip avance, dent après dent. Nino souffle, les épaules baissent. C'est à toi, Nino. J'y glisse un pied. Chacun son tour, sur le tapis. La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4581,13 +4580,13 @@
         <is>
           <t>enfant-m|J'attends la fermeture.
 papa|Moi je l'ouvre, puis c'est toi.
-narrateur|Nino tient la lampe, sur le tissu.
-narrateur|La fermeture avance, tout seule d'abord.
-narrateur|Nino souffle, puis il recule.
+narrateur|Nino tient la lampe, le sac attend.
+narrateur|Le zip avance, dent après dent.
+narrateur|Nino souffle, les épaules baissent.
 papa|C'est à toi, Nino.
-enfant-m|Merci, j'y vais.
+enfant-m|J'y glisse un pied.
 maman|Chacun son tour, sur le tapis.
-narrateur|L'élan a attendu la place.</t>
+narrateur|La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
     </row>
@@ -4614,12 +4613,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le bout du tapis attend encore, tout lisse. J'ai ouvert, puis c'était toi. J'ai attendu ta place. Chacun son tour, sur le tissu. L'élan a laissé la place. La lampe torche garde un grain de poussière. Nino souffle dessus, tout doux. On se dit au revoir, tapis. Un fil oublié sèche contre le pied.</t>
+          <t>Nino s'allonge dans le sac ouvert. J'ai ouvert, puis c'était toi. J'ai attendu le zip. Chacun son tour, sur le tapis. La tente verte tient, enfin. La lampe torche garde un grain de poussière. Nino souffle dessus, tout doux. Bonne nuit, tapis. Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Le bout du tapis attend encore, tout lisse. J'ai ouvert, puis c'était toi. J'ai attendu ta place. Chacun son tour, sur le tissu. L'élan a laissé la place. La lampe torche garde un grain de poussière. Nino souffle dessus, tout doux. On se dit au revoir, tapis. Un fil oublié sèche contre le pied.</t>
+          <t>Nino s'allonge dans le sac ouvert. J'ai ouvert, puis c'était toi. J'ai attendu le zip. Chacun son tour, sur le tapis. La tente verte tient, enfin. La lampe torche garde un grain de poussière. Nino souffle dessus, tout doux. Bonne nuit, tapis. Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4754,14 +4753,14 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Le bout du tapis attend encore, tout lisse.
+          <t>narrateur|Nino s'allonge dans le sac ouvert.
 papa|J'ai ouvert, puis c'était toi.
-enfant-m|J'ai attendu ta place.
-maman|Chacun son tour, sur le tissu.
-narrateur|L'élan a laissé la place.
+enfant-m|J'ai attendu le zip.
+maman|Chacun son tour, sur le tapis.
+narrateur|La tente verte tient, enfin.
 narrateur|La lampe torche garde un grain de poussière.
 narrateur|Nino souffle dessus, tout doux.
-enfant-m|On se dit au revoir, tapis.
+enfant-m|Bonne nuit, tapis.
 narrateur|Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
@@ -4789,12 +4788,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de la lampe. Nino glisse un pied, et ses genoux se posent. L'autre pied suit, la lampe au calme. On demande, et ça va juste. Vous avez demandé, et ça marche. Le sac a tenu l'élan. Un carré de tapis reste tiède, autour.</t>
+          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de la lampe. Nino glisse un pied, les genoux se posent. L'autre pied suit, la lampe au calme. Toi tu ouvres, moi j'entre. Vous avez demandé, et ça marche. Le sac tient tout seul, maintenant. Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de la lampe. Nino glisse un pied, et ses genoux se posent. L'autre pied suit, la lampe au calme. On demande, et ça va juste. Vous avez demandé, et ça marche. Le sac a tenu l'élan. Un carré de tapis reste tiède, autour.</t>
+          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de la lampe. Nino glisse un pied, les genoux se posent. L'autre pied suit, la lampe au calme. Toi tu ouvres, moi j'entre. Vous avez demandé, et ça marche. Le sac tient tout seul, maintenant. Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4932,11 +4931,11 @@
           <t>enfant-m|Papa, tu ouvres le sac ?
 papa|Je l'ouvre, tout doux.
 narrateur|Papa ouvre le sac près de la lampe.
-narrateur|Nino glisse un pied, et ses genoux se posent.
+narrateur|Nino glisse un pied, les genoux se posent.
 narrateur|L'autre pied suit, la lampe au calme.
-enfant-m|On demande, et ça va juste.
+enfant-m|Toi tu ouvres, moi j'entre.
 maman|Vous avez demandé, et ça marche.
-papa|Le sac a tenu l'élan.
+papa|Le sac tient tout seul, maintenant.
 narrateur|Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
@@ -4964,12 +4963,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Le sac de papa repose sur le tapis. Tu l'ouvrais, tout grand. On a demandé, et ça allait juste. L'ouverture a fait le tour, rien de plus. Le tapis a rendu le calme. La lampe torche garde un rond tiède, tout petit. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
+          <t>Nino s'allonge, le sac ouvert par papa. Tu l'ouvrais, tout grand. Le sac s'est ouvert, juste assez. L'entrée du camp est à vous. Le tapis a rendu le calme. La lampe torche garde un rond tiède, tout petit. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Le sac de papa repose sur le tapis. Tu l'ouvrais, tout grand. On a demandé, et ça allait juste. L'ouverture a fait le tour, rien de plus. Le tapis a rendu le calme. La lampe torche garde un rond tiède, tout petit. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
+          <t>Nino s'allonge, le sac ouvert par papa. Tu l'ouvrais, tout grand. Le sac s'est ouvert, juste assez. L'entrée du camp est à vous. Le tapis a rendu le calme. La lampe torche garde un rond tiède, tout petit. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5104,10 +5103,10 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|Le sac de papa repose sur le tapis.
+          <t>narrateur|Nino s'allonge, le sac ouvert par papa.
 enfant-m|Tu l'ouvrais, tout grand.
-papa|On a demandé, et ça allait juste.
-maman|L'ouverture a fait le tour, rien de plus.
+papa|Le sac s'est ouvert, juste assez.
+maman|L'entrée du camp est à vous.
 narrateur|Le tapis a rendu le calme.
 narrateur|La lampe torche garde un rond tiède, tout petit.
 narrateur|Un rond de chaleur reste sur le tissu.
@@ -5139,12 +5138,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>La lampe torche pose son rond au pied du lit. Ici, ça mène au camp, papa. Le bois du lit renvoie chaque pas, tout fort. Les sauts de Nino chassent le rond, trop haut. La lampe torche attend au bord, un peu seule. Son élan remplit tout le lit. Toi tu vas plus haut, trop vite. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Nino glisse la lampe au pied du lit. Ici, c'est la grotte, papa. Le bois du lit renvoie chaque pas. Le rond grimpe au bois, trop haut, trop vite. La lampe torche n'est plus à sa place. Tes genoux font trop de vagues. Le camp n'a pas encore de toit. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>La lampe torche pose son rond au pied du lit. Ici, ça mène au camp, papa. Le bois du lit renvoie chaque pas, tout fort. Les sauts de Nino chassent le rond, trop haut. La lampe torche attend au bord, un peu seule. Son élan remplit tout le lit. Toi tu vas plus haut, trop vite. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Nino glisse la lampe au pied du lit. Ici, c'est la grotte, papa. Le bois du lit renvoie chaque pas. Le rond grimpe au bois, trop haut, trop vite. La lampe torche n'est plus à sa place. Tes genoux font trop de vagues. Le camp n'a pas encore de toit. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5279,13 +5278,13 @@
       <c r="AV24" s="2" t="inlineStr"/>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>narrateur|La lampe torche pose son rond au pied du lit.
-enfant-m|Ici, ça mène au camp, papa.
-narrateur|Le bois du lit renvoie chaque pas, tout fort.
-narrateur|Les sauts de Nino chassent le rond, trop haut.
-narrateur|La lampe torche attend au bord, un peu seule.
-maman|Son élan remplit tout le lit.
-papa|Toi tu vas plus haut, trop vite.
+          <t>narrateur|Nino glisse la lampe au pied du lit.
+enfant-m|Ici, c'est la grotte, papa.
+narrateur|Le bois du lit renvoie chaque pas.
+narrateur|Le rond grimpe au bois, trop haut, trop vite.
+narrateur|La lampe torche n'est plus à sa place.
+maman|Tes genoux font trop de vagues.
+papa|Le camp n'a pas encore de toit.
 enfant-m|On s'allonge comment, alors ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -5314,12 +5313,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore au pied du lit. Les vagues, le matelas, ou maman ?</t>
+          <t>Le bois du lit tremble encore un peu. Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore au pied du lit. Les vagues, le matelas, ou maman ?</t>
+          <t>Le bois du lit tremble encore un peu. Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -5478,7 +5477,7 @@
       <c r="AV25" s="2" t="inlineStr"/>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|Nino rebondit encore au pied du lit.
+          <t>narrateur|Le bois du lit tremble encore un peu.
 papa|Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
@@ -5506,12 +5505,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. La lampe torche voyage d'un genou à l'autre. Ils avancent au pied du lit, l'un après l'autre. Doucement, les vagues tiennent. Vous jouez avec l'élan, ensemble. Le bois est devenu une rive. La lampe torche a fait le tour, sans se taire. Le camp est là, tout bas.</t>
+          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. La lampe voyage d'un genou à l'autre. Le bois devient une mer, puis une rive. Doucement, les vagues tiennent. Vous avez joué, puis calmé le lit. Le pied du lit est une grotte. La lampe torche a trouvé son coin. Le camp est là, tout bas.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. La lampe torche voyage d'un genou à l'autre. Ils avancent au pied du lit, l'un après l'autre. Doucement, les vagues tiennent. Vous jouez avec l'élan, ensemble. Le bois est devenu une rive. La lampe torche a fait le tour, sans se taire. Le camp est là, tout bas.</t>
+          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. La lampe voyage d'un genou à l'autre. Le bois devient une mer, puis une rive. Doucement, les vagues tiennent. Vous avez joué, puis calmé le lit. Le pied du lit est une grotte. La lampe torche a trouvé son coin. Le camp est là, tout bas.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5648,12 +5647,12 @@
         <is>
           <t>enfant-m|On fait des vagues.
 papa|Tu rebondis, puis tu t'arrêtes.
-narrateur|La lampe torche voyage d'un genou à l'autre.
-narrateur|Ils avancent au pied du lit, l'un après l'autre.
+narrateur|La lampe voyage d'un genou à l'autre.
+narrateur|Le bois devient une mer, puis une rive.
 enfant-m|Doucement, les vagues tiennent.
-maman|Vous jouez avec l'élan, ensemble.
-papa|Le bois est devenu une rive.
-narrateur|La lampe torche a fait le tour, sans se taire.
+maman|Vous avez joué, puis calmé le lit.
+papa|Le pied du lit est une grotte.
+narrateur|La lampe torche a trouvé son coin.
 enfant-m|Le camp est là, tout bas.</t>
         </is>
       </c>
@@ -5681,12 +5680,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Les vagues s'arrêtent contre le pied du lit. On est arrivés, tous les deux. Tu rebondissais, puis tu t'arrêtais. Le bois est redevenu un lit, simplement. L'élan s'est couché. La lampe torche garde un rond tiède, tout petit. Une poussière tourne encore, puis tombe. On s'allonge, les vagues se taisent. Dans la chambre, le camp redevient calme.</t>
+          <t>Nino s'allonge au pied du lit. Les vagues sont finies, papa. Tu rebondissais, puis tu t'arrêtais. La grotte a son camp, ce soir. Le bois est redevenu un lit. La lampe torche garde un rond tiède, tout petit. Une poussière tourne encore, puis tombe. Les vagues se taisent. Dans la chambre, le camp tient.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Les vagues s'arrêtent contre le pied du lit. On est arrivés, tous les deux. Tu rebondissais, puis tu t'arrêtais. Le bois est redevenu un lit, simplement. L'élan s'est couché. La lampe torche garde un rond tiède, tout petit. Une poussière tourne encore, puis tombe. On s'allonge, les vagues se taisent. Dans la chambre, le camp redevient calme.</t>
+          <t>Nino s'allonge au pied du lit. Les vagues sont finies, papa. Tu rebondissais, puis tu t'arrêtais. La grotte a son camp, ce soir. Le bois est redevenu un lit. La lampe torche garde un rond tiède, tout petit. Une poussière tourne encore, puis tombe. Les vagues se taisent. Dans la chambre, le camp tient.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5821,15 +5820,15 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|Les vagues s'arrêtent contre le pied du lit.
-enfant-m|On est arrivés, tous les deux.
+          <t>narrateur|Nino s'allonge au pied du lit.
+enfant-m|Les vagues sont finies, papa.
 papa|Tu rebondissais, puis tu t'arrêtais.
-maman|Le bois est redevenu un lit, simplement.
-narrateur|L'élan s'est couché.
+maman|La grotte a son camp, ce soir.
+narrateur|Le bois est redevenu un lit.
 narrateur|La lampe torche garde un rond tiède, tout petit.
 narrateur|Une poussière tourne encore, puis tombe.
-enfant-m|On s'allonge, les vagues se taisent.
-narrateur|Dans la chambre, le camp redevient calme.</t>
+enfant-m|Les vagues se taisent.
+narrateur|Dans la chambre, le camp tient.</t>
         </is>
       </c>
     </row>
@@ -5856,12 +5855,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. La lampe torche reste muette, au creux. Le matelas se tait, enfin. Maintenant ! Vous avez laissé le bois s'ouvrir. L'élan a attendu le pied. Un pli du drap retombe, tout lent.</t>
+          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. La lampe reste éteinte, au creux du sac. Le matelas se tait, enfin. Maintenant ! Le lit a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. La lampe torche reste muette, au creux. Le matelas se tait, enfin. Maintenant ! Vous avez laissé le bois s'ouvrir. L'élan a attendu le pied. Un pli du drap retombe, tout lent.</t>
+          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. La lampe reste éteinte, au creux du sac. Le matelas se tait, enfin. Maintenant ! Le lit a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -5999,11 +5998,11 @@
           <t>enfant-m|On attend le matelas.
 papa|Quand il se tait, tu t'allonges.
 narrateur|Un saut, puis le bois reste calme.
-narrateur|La lampe torche reste muette, au creux.
+narrateur|La lampe reste éteinte, au creux du sac.
 narrateur|Le matelas se tait, enfin.
 enfant-m|Maintenant !
-maman|Vous avez laissé le bois s'ouvrir.
-papa|L'élan a attendu le pied.
+maman|Le lit a fini ses vagues.
+papa|Tes genoux se sont assis, eux aussi.
 narrateur|Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
@@ -6031,12 +6030,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Le matelas s'est tu, enfin, tout à fait. On a attendu le bois. Quand il était calme, on s'allongeait. Le pied vous a laissé le sac. L'élan a écouté le bois. La lampe torche ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
+          <t>Nino s'allonge, le matelas tout calme. On a attendu le bois. Quand il s'est tu, tu es entré. Le pied du lit a fait un toit. Tes genoux se sont assis. La lampe torche ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Le matelas s'est tu, enfin, tout à fait. On a attendu le bois. Quand il était calme, on s'allongeait. Le pied vous a laissé le sac. L'élan a écouté le bois. La lampe torche ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
+          <t>Nino s'allonge, le matelas tout calme. On a attendu le bois. Quand il s'est tu, tu es entré. Le pied du lit a fait un toit. Tes genoux se sont assis. La lampe torche ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6171,11 +6170,11 @@
       <c r="AV29" s="2" t="inlineStr"/>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>narrateur|Le matelas s'est tu, enfin, tout à fait.
+          <t>narrateur|Nino s'allonge, le matelas tout calme.
 enfant-m|On a attendu le bois.
-papa|Quand il était calme, on s'allongeait.
-maman|Le pied vous a laissé le sac.
-narrateur|L'élan a écouté le bois.
+papa|Quand il s'est tu, tu es entré.
+maman|Le pied du lit a fait un toit.
+narrateur|Tes genoux se sont assis.
 narrateur|La lampe torche ne fait plus aucun bruit.
 narrateur|Nino pose la paume sur le bois tiède.
 enfant-m|Il est tiède.
@@ -6206,12 +6205,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac quand Nino tient la lampe. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit se range derrière le sac. Vous avez demandé le bord. Mes mains ont tenu l'élan.</t>
+          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac, Nino tient la lampe. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit devient un toit. Vous avez demandé le bord. Mes mains ont tenu le camp.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac quand Nino tient la lampe. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit se range derrière le sac. Vous avez demandé le bord. Mes mains ont tenu l'élan.</t>
+          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac, Nino tient la lampe. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit devient un toit. Vous avez demandé le bord. Mes mains ont tenu le camp.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -6348,13 +6347,13 @@
         <is>
           <t>enfant-m|Maman, tu bordes le sac ?
 maman|Je le borde, tout chaud.
-narrateur|Maman borde le sac quand Nino tient la lampe.
+narrateur|Maman borde le sac, Nino tient la lampe.
 narrateur|Nino écoute les mains, plus que ses pieds.
 papa|Tu t'allonges, et ça tient.
 enfant-m|Moi aussi, j'écoute.
-narrateur|Le pied du lit se range derrière le sac.
+narrateur|Le pied du lit devient un toit.
 papa|Vous avez demandé le bord.
-maman|Mes mains ont tenu l'élan.</t>
+maman|Mes mains ont tenu le camp.</t>
         </is>
       </c>
     </row>
@@ -6381,12 +6380,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Les mains de maman s'éteignent, un à un. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. La lampe torche garde un rond tiède, tout petit. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
+          <t>Nino s'allonge, le sac bordé par maman. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. La lampe torche garde un rond tiède, tout petit. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Les mains de maman s'éteignent, un à un. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. La lampe torche garde un rond tiède, tout petit. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
+          <t>Nino s'allonge, le sac bordé par maman. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. La lampe torche garde un rond tiède, tout petit. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6521,7 +6520,7 @@
       <c r="AV31" s="2" t="inlineStr"/>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>narrateur|Les mains de maman s'éteignent, un à un.
+          <t>narrateur|Nino s'allonge, le sac bordé par maman.
 enfant-m|J'écoutais tes mains.
 papa|Moi aussi, je bordais avec toi.
 maman|Vous avez demandé le bord.
@@ -6916,12 +6915,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Sous le bras. Oui. Le sac vert tient une ombre longue. On le pose pour la nuit. Nino a les cheveux tout droits, encore. Une mèche saute quand il respire. Ça sent déjà le tapis tiède. Tes mains, sur le sac ? Oui, papa.</t>
+          <t>Sous le bras. Oui. La fermeture du sac chatouille sa manche. C'est ma tente, pour ce soir. Nino secoue le sac, un nuage de coton. Un coin vert traîne encore par terre. Ça sent le linge tiède, déjà. Tes mains, sur le sac ? Oui, papa.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Sous le bras. Oui. Le sac vert tient une ombre longue. On le pose pour la nuit. Nino a les cheveux tout droits, encore. Une mèche saute quand il respire. Ça sent déjà le tapis tiède. Tes mains, sur le sac ? Oui, papa.</t>
+          <t>Sous le bras. Oui. La fermeture du sac chatouille sa manche. C'est ma tente, pour ce soir. Nino secoue le sac, un nuage de coton. Un coin vert traîne encore par terre. Ça sent le linge tiède, déjà. Tes mains, sur le sac ? Oui, papa.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7062,11 +7061,11 @@
         <is>
           <t>enfant-m|Sous le bras.
 papa|Oui.
-narrateur|Le sac vert tient une ombre longue.
-enfant-m|On le pose pour la nuit.
-narrateur|Nino a les cheveux tout droits, encore.
-narrateur|Une mèche saute quand il respire.
-maman|Ça sent déjà le tapis tiède.
+narrateur|La fermeture du sac chatouille sa manche.
+enfant-m|C'est ma tente, pour ce soir.
+narrateur|Nino secoue le sac, un nuage de coton.
+narrateur|Un coin vert traîne encore par terre.
+maman|Ça sent le linge tiède, déjà.
 papa|Tes mains, sur le sac ?
 enfant-m|Oui, papa.</t>
         </is>
@@ -7095,12 +7094,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Nino tapote déjà le parquet, tout léger. La fenêtre garde un rai de rue. Le tapis fait un carré chaud. Le pied du lit attend, tout bas. On campe où, Nino ?</t>
+          <t>Nino tapote déjà le parquet, tout léger. Sous la fenêtre, le rideau garde un rai de rue. Au milieu, le tapis fait un carré chaud. Près du bois, le pied du lit attend. On campe où, Nino ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Nino tapote déjà le parquet, tout léger. La fenêtre garde un rai de rue. Le tapis fait un carré chaud. Le pied du lit attend, tout bas. On campe où, Nino ?</t>
+          <t>Nino tapote déjà le parquet, tout léger. Sous la fenêtre, le rideau garde un rai de rue. Au milieu, le tapis fait un carré chaud. Près du bois, le pied du lit attend. On campe où, Nino ?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -7260,9 +7259,9 @@
       <c r="AW35" t="inlineStr">
         <is>
           <t>narrateur|Nino tapote déjà le parquet, tout léger.
-narrateur|La fenêtre garde un rai de rue.
-narrateur|Le tapis fait un carré chaud.
-narrateur|Le pied du lit attend, tout bas.
+narrateur|Sous la fenêtre, le rideau garde un rai de rue.
+narrateur|Au milieu, le tapis fait un carré chaud.
+narrateur|Près du bois, le pied du lit attend.
 papa|On campe où, Nino ?</t>
         </is>
       </c>
@@ -7290,12 +7289,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Le sac vert penche vers la fenêtre. Nino tape le parquet, trop vite. Moi je cours, papa ! Ses pieds font des ronds, trop larges. Le sac tape le bois, un choc trop sec. Le sac vert n'attendait pas ça. Il a envie de bouger, c'est tout. Tes jambes sont plus vives, ce soir. On campe comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Nino traîne le sac vers le rideau. Ses talons tambourinent le parquet. Le camp, c'est là, papa ! Le sac cogne le rebord, clic trop fort. Le sac vert part trop vite. Tes pieds dansent, ce soir. Le rideau n'est pas encore une tente. On campe comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Le sac vert penche vers la fenêtre. Nino tape le parquet, trop vite. Moi je cours, papa ! Ses pieds font des ronds, trop larges. Le sac tape le bois, un choc trop sec. Le sac vert n'attendait pas ça. Il a envie de bouger, c'est tout. Tes jambes sont plus vives, ce soir. On campe comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Nino traîne le sac vers le rideau. Ses talons tambourinent le parquet. Le camp, c'est là, papa ! Le sac cogne le rebord, clic trop fort. Le sac vert part trop vite. Tes pieds dansent, ce soir. Le rideau n'est pas encore une tente. On campe comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7430,14 +7429,13 @@
       <c r="AV36" s="2" t="inlineStr"/>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>narrateur|Le sac vert penche vers la fenêtre.
-narrateur|Nino tape le parquet, trop vite.
-enfant-m|Moi je cours, papa !
-narrateur|Ses pieds font des ronds, trop larges.
-narrateur|Le sac tape le bois, un choc trop sec.
-enfant-m|Le sac vert n'attendait pas ça.
-maman|Il a envie de bouger, c'est tout.
-papa|Tes jambes sont plus vives, ce soir.
+          <t>narrateur|Nino traîne le sac vers le rideau.
+narrateur|Ses talons tambourinent le parquet.
+enfant-m|Le camp, c'est là, papa !
+narrateur|Le sac cogne le rebord, clic trop fort.
+enfant-m|Le sac vert part trop vite.
+maman|Tes pieds dansent, ce soir.
+papa|Le rideau n'est pas encore une tente.
 enfant-m|On campe comment, alors ?
 papa|Tu fais comment, avec nous ?</t>
         </is>
@@ -7466,12 +7464,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Nino tape encore le parquet, tout fort. Les lucioles, le rideau, ou maman ?</t>
+          <t>Le lapin de lumière court encore. Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Nino tape encore le parquet, tout fort. Les lucioles, le rideau, ou maman ?</t>
+          <t>Le lapin de lumière court encore. Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -7630,7 +7628,7 @@
       <c r="AV37" s="2" t="inlineStr"/>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|Nino tape encore le parquet, tout fort.
+          <t>narrateur|Le lapin de lumière court encore.
 papa|Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
@@ -7658,12 +7656,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>On joue aux lucioles. Toi tu bouges, moi je suis le rond. Nino tient le sac, le faisceau danse. Deux ronds se croisent sur le rideau. Nino saute une fois, puis s'arrête. Maintenant c'est le camp. L'élan a trouvé sa fenêtre. Vous jouez à tour, sur le tissu. Le rideau redevient un mur, tout doux.</t>
+          <t>On joue aux lucioles. Toi tu clignes, moi je compte. Nino cligne, le sac devient une colline. Des points d'or s'allument sur le rideau. Nino cligne encore, puis s'arrête. Les lucioles sont fatiguées. Le camp a sa lumière, maintenant. Vous avez dansé, puis posé. Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>On joue aux lucioles. Toi tu bouges, moi je suis le rond. Nino tient le sac, le faisceau danse. Deux ronds se croisent sur le rideau. Nino saute une fois, puis s'arrête. Maintenant c'est le camp. L'élan a trouvé sa fenêtre. Vous jouez à tour, sur le tissu. Le rideau redevient un mur, tout doux.</t>
+          <t>On joue aux lucioles. Toi tu clignes, moi je compte. Nino cligne, le sac devient une colline. Des points d'or s'allument sur le rideau. Nino cligne encore, puis s'arrête. Les lucioles sont fatiguées. Le camp a sa lumière, maintenant. Vous avez dansé, puis posé. Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7799,14 +7797,14 @@
       <c r="AW38" t="inlineStr">
         <is>
           <t>enfant-m|On joue aux lucioles.
-papa|Toi tu bouges, moi je suis le rond.
-narrateur|Nino tient le sac, le faisceau danse.
-narrateur|Deux ronds se croisent sur le rideau.
-narrateur|Nino saute une fois, puis s'arrête.
-enfant-m|Maintenant c'est le camp.
-maman|L'élan a trouvé sa fenêtre.
-papa|Vous jouez à tour, sur le tissu.
-narrateur|Le rideau redevient un mur, tout doux.</t>
+papa|Toi tu clignes, moi je compte.
+narrateur|Nino cligne, le sac devient une colline.
+narrateur|Des points d'or s'allument sur le rideau.
+narrateur|Nino cligne encore, puis s'arrête.
+enfant-m|Les lucioles sont fatiguées.
+maman|Le camp a sa lumière, maintenant.
+papa|Vous avez dansé, puis posé.
+narrateur|Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
     </row>
@@ -7833,12 +7831,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le dernier rond du rideau est à eux. On a joué, chacun son tour. Toi tu bougais, moi je suivais. Vous avez laissé l'élan dessiner. La chambre sent encore le savon. Le sac vert garde un pli chaud, près de la fermeture. Un trait clair dort sur le bois. On s'allonge, papa. Les chaussettes retrouvent le tapis tiède.</t>
+          <t>Nino s'allonge, le sac sous le rideau. Les lucioles sont couchées, papa. Toi tu clignais, moi je comptais. Le camp a sa lumière, ce soir. La chambre sent encore le savon. Le sac vert garde un pli chaud, près de la fermeture. Un point d'or dort sur le tissu. Bonne nuit, fenêtre. Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Le dernier rond du rideau est à eux. On a joué, chacun son tour. Toi tu bougais, moi je suivais. Vous avez laissé l'élan dessiner. La chambre sent encore le savon. Le sac vert garde un pli chaud, près de la fermeture. Un trait clair dort sur le bois. On s'allonge, papa. Les chaussettes retrouvent le tapis tiède.</t>
+          <t>Nino s'allonge, le sac sous le rideau. Les lucioles sont couchées, papa. Toi tu clignais, moi je comptais. Le camp a sa lumière, ce soir. La chambre sent encore le savon. Le sac vert garde un pli chaud, près de la fermeture. Un point d'or dort sur le tissu. Bonne nuit, fenêtre. Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7973,14 +7971,14 @@
       <c r="AV39" s="2" t="inlineStr"/>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|Le dernier rond du rideau est à eux.
-enfant-m|On a joué, chacun son tour.
-papa|Toi tu bougais, moi je suivais.
-maman|Vous avez laissé l'élan dessiner.
+          <t>narrateur|Nino s'allonge, le sac sous le rideau.
+enfant-m|Les lucioles sont couchées, papa.
+papa|Toi tu clignais, moi je comptais.
+maman|Le camp a sa lumière, ce soir.
 narrateur|La chambre sent encore le savon.
 narrateur|Le sac vert garde un pli chaud, près de la fermeture.
-narrateur|Un trait clair dort sur le bois.
-enfant-m|On s'allonge, papa.
+narrateur|Un point d'or dort sur le tissu.
+enfant-m|Bonne nuit, fenêtre.
 narrateur|Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
@@ -8008,12 +8006,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu. Nino pose les genoux au bois. Le sac vert attend près du rebord. Sa respiration redevient calme, tout doux. Je suis prêt ? Le rideau ne bouge plus. Vous avez laissé l'élan s'asseoir. Le faisceau tient enfin, tout droit. Le camp peut s'ouvrir.</t>
+          <t>On attend le rideau. Nino pose les genoux au parquet. Le sac repose contre le rebord, plié. Le volet tape une fois, puis plus. Il ne bouge plus ? Le tissu est calme, oui. Tes pieds se sont assis, eux aussi. Nino rallume, tout droit, tout petit. Le camp peut s'ouvrir.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu. Nino pose les genoux au bois. Le sac vert attend près du rebord. Sa respiration redevient calme, tout doux. Je suis prêt ? Le rideau ne bouge plus. Vous avez laissé l'élan s'asseoir. Le faisceau tient enfin, tout droit. Le camp peut s'ouvrir.</t>
+          <t>On attend le rideau. Nino pose les genoux au parquet. Le sac repose contre le rebord, plié. Le volet tape une fois, puis plus. Il ne bouge plus ? Le tissu est calme, oui. Tes pieds se sont assis, eux aussi. Nino rallume, tout droit, tout petit. Le camp peut s'ouvrir.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8148,14 +8146,14 @@
       <c r="AV40" s="2" t="inlineStr"/>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>enfant-m|On attend un peu.
-narrateur|Nino pose les genoux au bois.
-narrateur|Le sac vert attend près du rebord.
-narrateur|Sa respiration redevient calme, tout doux.
-enfant-m|Je suis prêt ?
-maman|Le rideau ne bouge plus.
-papa|Vous avez laissé l'élan s'asseoir.
-narrateur|Le faisceau tient enfin, tout droit.
+          <t>enfant-m|On attend le rideau.
+narrateur|Nino pose les genoux au parquet.
+narrateur|Le sac repose contre le rebord, plié.
+narrateur|Le volet tape une fois, puis plus.
+enfant-m|Il ne bouge plus ?
+maman|Le tissu est calme, oui.
+papa|Tes pieds se sont assis, eux aussi.
+narrateur|Nino rallume, tout droit, tout petit.
 enfant-m|Le camp peut s'ouvrir.</t>
         </is>
       </c>
@@ -8183,12 +8181,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le rebord de la fenêtre garde encore la chaleur. Je me suis arrêté, d'abord. Puis le faisceau est resté droit. L'élan s'est assis, puis il a campé. Le rideau redevient calme. Le sac vert garde un pli chaud, près de la fermeture. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
+          <t>Nino s'allonge, le rideau tout calme. J'ai attendu le volet, d'abord. Puis le faisceau est resté droit. Tes pieds se sont assis, eux aussi. Le tissu ne danse plus. Le sac vert garde un pli chaud, près de la fermeture. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Le rebord de la fenêtre garde encore la chaleur. Je me suis arrêté, d'abord. Puis le faisceau est resté droit. L'élan s'est assis, puis il a campé. Le rideau redevient calme. Le sac vert garde un pli chaud, près de la fermeture. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
+          <t>Nino s'allonge, le rideau tout calme. J'ai attendu le volet, d'abord. Puis le faisceau est resté droit. Tes pieds se sont assis, eux aussi. Le tissu ne danse plus. Le sac vert garde un pli chaud, près de la fermeture. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8323,11 +8321,11 @@
       <c r="AV41" s="2" t="inlineStr"/>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Le rebord de la fenêtre garde encore la chaleur.
-enfant-m|Je me suis arrêté, d'abord.
+          <t>narrateur|Nino s'allonge, le rideau tout calme.
+enfant-m|J'ai attendu le volet, d'abord.
 papa|Puis le faisceau est resté droit.
-maman|L'élan s'est assis, puis il a campé.
-narrateur|Le rideau redevient calme.
+maman|Tes pieds se sont assis, eux aussi.
+narrateur|Le tissu ne danse plus.
 narrateur|Le sac vert garde un pli chaud, près de la fermeture.
 narrateur|Une poussière reste coincée, tout près.
 enfant-m|À demain, les ronds.
@@ -8358,12 +8356,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens la lampe ? Je la tiens, un pas chacun. Maman pose le sac près de sa main. Nino pose un pied, puis l'autre. Le faisceau reste sage, juste à côté. On demande, et ça va ! Vous avez demandé, tout calme. Ma main a juste attendu. La fenêtre garde un rai, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu poses le camp. Maman tient le sac, Nino tend la lampe. Nino étale le sac sous le rai de rue. Le faisceau reste sage, dans sa main. Toi tu tiens, moi je range. Vous avez demandé, et ça tient. Ma main fait le piquet, ce soir. La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens la lampe ? Je la tiens, un pas chacun. Maman pose le sac près de sa main. Nino pose un pied, puis l'autre. Le faisceau reste sage, juste à côté. On demande, et ça va ! Vous avez demandé, tout calme. Ma main a juste attendu. La fenêtre garde un rai, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu poses le camp. Maman tient le sac, Nino tend la lampe. Nino étale le sac sous le rai de rue. Le faisceau reste sage, dans sa main. Toi tu tiens, moi je range. Vous avez demandé, et ça tient. Ma main fait le piquet, ce soir. La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8498,14 +8496,14 @@
       <c r="AV42" s="2" t="inlineStr"/>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>enfant-m|Maman, tu tiens la lampe ?
-maman|Je la tiens, un pas chacun.
-narrateur|Maman pose le sac près de sa main.
-narrateur|Nino pose un pied, puis l'autre.
-narrateur|Le faisceau reste sage, juste à côté.
-enfant-m|On demande, et ça va !
-papa|Vous avez demandé, tout calme.
-maman|Ma main a juste attendu.
+          <t>enfant-m|Maman, tu tiens, s'il te plaît ?
+maman|Je tiens, tu poses le camp.
+narrateur|Maman tient le sac, Nino tend la lampe.
+narrateur|Nino étale le sac sous le rai de rue.
+narrateur|Le faisceau reste sage, dans sa main.
+enfant-m|Toi tu tiens, moi je range.
+papa|Vous avez demandé, et ça tient.
+maman|Ma main fait le piquet, ce soir.
 narrateur|La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
@@ -8533,12 +8531,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>La main de maman reste dans l'air, tout légère. J'ai attendu le pas. On a demandé, et ça allait. Sa main a tenu vos pieds. La chambre vous rend le silence. Le sac vert pose un grain de lumière sur le bois. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
+          <t>Nino s'allonge, la main de maman tout près. Tu tenais le piquet. Vous avez demandé, et ça tenait. Ma main a fait la tente. La chambre rend le silence, tout doux. Le sac vert pose un grain de lumière. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>La main de maman reste dans l'air, tout légère. J'ai attendu le pas. On a demandé, et ça allait. Sa main a tenu vos pieds. La chambre vous rend le silence. Le sac vert pose un grain de lumière sur le bois. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
+          <t>Nino s'allonge, la main de maman tout près. Tu tenais le piquet. Vous avez demandé, et ça tenait. Ma main a fait la tente. La chambre rend le silence, tout doux. Le sac vert pose un grain de lumière. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8673,12 +8671,12 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|La main de maman reste dans l'air, tout légère.
-enfant-m|J'ai attendu le pas.
-papa|On a demandé, et ça allait.
-maman|Sa main a tenu vos pieds.
-narrateur|La chambre vous rend le silence.
-narrateur|Le sac vert pose un grain de lumière sur le bois.
+          <t>narrateur|Nino s'allonge, la main de maman tout près.
+enfant-m|Tu tenais le piquet.
+papa|Vous avez demandé, et ça tenait.
+maman|Ma main a fait la tente.
+narrateur|La chambre rend le silence, tout doux.
+narrateur|Le sac vert pose un grain de lumière.
 narrateur|Nino touche le rideau, du bout.
 enfant-m|Il est à nous.
 narrateur|Un rai de rue barre encore le tissu.</t>
@@ -8708,12 +8706,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Le sac vert glisse au milieu du tapis. Le tapis est à nous, maman. Ses pieds quittent le tissu, puis reviennent. Nino rebondit, le sac part trop loin. Un peu de poussière lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, trop vite. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Nino déroule le sac au milieu du tapis. Ici, c'est la clairière, maman. Ses genoux font un petit trampoline. Le sac glisse comme un escargot trop pressé. Un fil de laine se lève, puis retombe. Ton corps veut encore courir. Le tapis n'a pas encore de tente. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Le sac vert glisse au milieu du tapis. Le tapis est à nous, maman. Ses pieds quittent le tissu, puis reviennent. Nino rebondit, le sac part trop loin. Un peu de poussière lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, trop vite. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Nino déroule le sac au milieu du tapis. Ici, c'est la clairière, maman. Ses genoux font un petit trampoline. Le sac glisse comme un escargot trop pressé. Un fil de laine se lève, puis retombe. Ton corps veut encore courir. Le tapis n'a pas encore de tente. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8848,13 +8846,13 @@
       <c r="AV44" s="2" t="inlineStr"/>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>narrateur|Le sac vert glisse au milieu du tapis.
-enfant-m|Le tapis est à nous, maman.
-narrateur|Ses pieds quittent le tissu, puis reviennent.
-narrateur|Nino rebondit, le sac part trop loin.
-narrateur|Un peu de poussière lève, puis retombe.
-maman|Il a de l'élan, comme un petit vent.
-papa|Toi tu vas plus loin, trop vite.
+          <t>narrateur|Nino déroule le sac au milieu du tapis.
+enfant-m|Ici, c'est la clairière, maman.
+narrateur|Ses genoux font un petit trampoline.
+narrateur|Le sac glisse comme un escargot trop pressé.
+narrateur|Un fil de laine se lève, puis retombe.
+maman|Ton corps veut encore courir.
+papa|Le tapis n'a pas encore de tente.
 enfant-m|On peut jouer avec, quand même ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -8883,12 +8881,12 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore sur le tapis. Le sentier, la fermeture, ou papa ?</t>
+          <t>Le sac n'a pas encore de forme. Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore sur le tapis. Le sentier, la fermeture, ou papa ?</t>
+          <t>Le sac n'a pas encore de forme. Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -9047,7 +9045,7 @@
       <c r="AV45" s="2" t="inlineStr"/>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|Nino rebondit encore sur le tapis.
+          <t>narrateur|Le sac n'a pas encore de forme.
 maman|Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
@@ -9075,12 +9073,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On fait un sentier. Toi derrière, moi devant ! Nino garde le sac, papa saute devant. Deux ombres passent sur le même tapis. Nino va plus vite, papa plus loin. On arrive au bout, tous les deux. Vous avez joué avec l'élan. Le tapis vous a laissés passer. Un fil de laine reste, tout petit.</t>
+          <t>On fait un sentier. Toi tu sautes, moi je suis derrière. Nino pose le sac, papa marque le sentier. Des pas dessinent un chemin sur le tapis. Nino saute une case, papa une autre. La clairière est au bout. Vous avez joué, puis posé le sac. Le tapis est devenu un chemin. Un fil de laine reste, tout petit.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>On fait un sentier. Toi derrière, moi devant ! Nino garde le sac, papa saute devant. Deux ombres passent sur le même tapis. Nino va plus vite, papa plus loin. On arrive au bout, tous les deux. Vous avez joué avec l'élan. Le tapis vous a laissés passer. Un fil de laine reste, tout petit.</t>
+          <t>On fait un sentier. Toi tu sautes, moi je suis derrière. Nino pose le sac, papa marque le sentier. Des pas dessinent un chemin sur le tapis. Nino saute une case, papa une autre. La clairière est au bout. Vous avez joué, puis posé le sac. Le tapis est devenu un chemin. Un fil de laine reste, tout petit.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9216,13 +9214,13 @@
       <c r="AW46" t="inlineStr">
         <is>
           <t>enfant-m|On fait un sentier.
-papa|Toi derrière, moi devant !
-narrateur|Nino garde le sac, papa saute devant.
-narrateur|Deux ombres passent sur le même tapis.
-narrateur|Nino va plus vite, papa plus loin.
-enfant-m|On arrive au bout, tous les deux.
-maman|Vous avez joué avec l'élan.
-papa|Le tapis vous a laissés passer.
+papa|Toi tu sautes, moi je suis derrière.
+narrateur|Nino pose le sac, papa marque le sentier.
+narrateur|Des pas dessinent un chemin sur le tapis.
+narrateur|Nino saute une case, papa une autre.
+enfant-m|La clairière est au bout.
+maman|Vous avez joué, puis posé le sac.
+papa|Le tapis est devenu un chemin.
 narrateur|Un fil de laine reste, tout petit.</t>
         </is>
       </c>
@@ -9250,12 +9248,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Deux paires de chaussettes marquent le bout du tapis. Toi devant, moi derrière. Tes jambes allaient plus loin. Vous avez sauté avec l'élan, pas contre. Le tapis redevient chaud, et calme. Le sac vert garde un pli chaud, près de la fermeture. Un peu de laine sèche déjà sur le tissu. On s'allonge, le sentier reste. Le lit fait une ombre longue.</t>
+          <t>Nino s'allonge au bout du sentier. Toi devant, moi derrière. Tes sauts ont fait le chemin. La clairière est devenue un camp. Le tapis redevient chaud, et calme. Le sac vert garde un pli chaud, près de la fermeture. Un peu de laine sèche déjà. Le sentier reste, maman. Le lit fait une ombre longue.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Deux paires de chaussettes marquent le bout du tapis. Toi devant, moi derrière. Tes jambes allaient plus loin. Vous avez sauté avec l'élan, pas contre. Le tapis redevient chaud, et calme. Le sac vert garde un pli chaud, près de la fermeture. Un peu de laine sèche déjà sur le tissu. On s'allonge, le sentier reste. Le lit fait une ombre longue.</t>
+          <t>Nino s'allonge au bout du sentier. Toi devant, moi derrière. Tes sauts ont fait le chemin. La clairière est devenue un camp. Le tapis redevient chaud, et calme. Le sac vert garde un pli chaud, près de la fermeture. Un peu de laine sèche déjà. Le sentier reste, maman. Le lit fait une ombre longue.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9390,14 +9388,14 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|Deux paires de chaussettes marquent le bout du tapis.
+          <t>narrateur|Nino s'allonge au bout du sentier.
 enfant-m|Toi devant, moi derrière.
-papa|Tes jambes allaient plus loin.
-maman|Vous avez sauté avec l'élan, pas contre.
+papa|Tes sauts ont fait le chemin.
+maman|La clairière est devenue un camp.
 narrateur|Le tapis redevient chaud, et calme.
 narrateur|Le sac vert garde un pli chaud, près de la fermeture.
-narrateur|Un peu de laine sèche déjà sur le tissu.
-enfant-m|On s'allonge, le sentier reste.
+narrateur|Un peu de laine sèche déjà.
+enfant-m|Le sentier reste, maman.
 narrateur|Le lit fait une ombre longue.</t>
         </is>
       </c>
@@ -9425,12 +9423,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient le sac, sur le tissu. La fermeture avance, tout seule d'abord. Nino souffle, puis il recule. C'est à toi, Nino. Merci, j'y vais. Chacun son tour, sur le tapis. L'élan a attendu la place.</t>
+          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient le sac, la fermeture attend. Le zip avance, dent après dent. Nino souffle, les épaules baissent. C'est à toi, Nino. J'y glisse un pied. Chacun son tour, sur le tapis. La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient le sac, sur le tissu. La fermeture avance, tout seule d'abord. Nino souffle, puis il recule. C'est à toi, Nino. Merci, j'y vais. Chacun son tour, sur le tapis. L'élan a attendu la place.</t>
+          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient le sac, la fermeture attend. Le zip avance, dent après dent. Nino souffle, les épaules baissent. C'est à toi, Nino. J'y glisse un pied. Chacun son tour, sur le tapis. La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9567,13 +9565,13 @@
         <is>
           <t>enfant-m|J'attends la fermeture.
 papa|Moi je l'ouvre, puis c'est toi.
-narrateur|Nino tient le sac, sur le tissu.
-narrateur|La fermeture avance, tout seule d'abord.
-narrateur|Nino souffle, puis il recule.
+narrateur|Nino tient le sac, la fermeture attend.
+narrateur|Le zip avance, dent après dent.
+narrateur|Nino souffle, les épaules baissent.
 papa|C'est à toi, Nino.
-enfant-m|Merci, j'y vais.
+enfant-m|J'y glisse un pied.
 maman|Chacun son tour, sur le tapis.
-narrateur|L'élan a attendu la place.</t>
+narrateur|La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
     </row>
@@ -9600,12 +9598,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le bout du tapis attend encore, tout lisse. J'ai ouvert, puis c'était toi. J'ai attendu ta place. Chacun son tour, sur le tissu. L'élan a laissé la place. Le sac vert garde un grain de poussière. Nino souffle dessus, tout doux. On se dit au revoir, tapis. Un fil oublié sèche contre le pied.</t>
+          <t>Nino s'allonge dans le sac ouvert. J'ai ouvert, puis c'était toi. J'ai attendu le zip. Chacun son tour, sur le tapis. La tente verte tient, enfin. Le sac vert garde un grain de poussière. Nino souffle dessus, tout doux. Bonne nuit, tapis. Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Le bout du tapis attend encore, tout lisse. J'ai ouvert, puis c'était toi. J'ai attendu ta place. Chacun son tour, sur le tissu. L'élan a laissé la place. Le sac vert garde un grain de poussière. Nino souffle dessus, tout doux. On se dit au revoir, tapis. Un fil oublié sèche contre le pied.</t>
+          <t>Nino s'allonge dans le sac ouvert. J'ai ouvert, puis c'était toi. J'ai attendu le zip. Chacun son tour, sur le tapis. La tente verte tient, enfin. Le sac vert garde un grain de poussière. Nino souffle dessus, tout doux. Bonne nuit, tapis. Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9740,14 +9738,14 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Le bout du tapis attend encore, tout lisse.
+          <t>narrateur|Nino s'allonge dans le sac ouvert.
 papa|J'ai ouvert, puis c'était toi.
-enfant-m|J'ai attendu ta place.
-maman|Chacun son tour, sur le tissu.
-narrateur|L'élan a laissé la place.
+enfant-m|J'ai attendu le zip.
+maman|Chacun son tour, sur le tapis.
+narrateur|La tente verte tient, enfin.
 narrateur|Le sac vert garde un grain de poussière.
 narrateur|Nino souffle dessus, tout doux.
-enfant-m|On se dit au revoir, tapis.
+enfant-m|Bonne nuit, tapis.
 narrateur|Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
@@ -9775,12 +9773,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac, tout grand. Nino glisse un pied, et ses genoux se posent. L'autre pied suit, la lampe au calme. On demande, et ça va juste. Vous avez demandé, et ça marche. Le sac a tenu l'élan. Un carré de tapis reste tiède, autour.</t>
+          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac, tout grand. Nino glisse un pied, les genoux se posent. L'autre pied suit, la lampe au calme. Toi tu ouvres, moi j'entre. Vous avez demandé, et ça marche. Le sac tient tout seul, maintenant. Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac, tout grand. Nino glisse un pied, et ses genoux se posent. L'autre pied suit, la lampe au calme. On demande, et ça va juste. Vous avez demandé, et ça marche. Le sac a tenu l'élan. Un carré de tapis reste tiède, autour.</t>
+          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac, tout grand. Nino glisse un pied, les genoux se posent. L'autre pied suit, la lampe au calme. Toi tu ouvres, moi j'entre. Vous avez demandé, et ça marche. Le sac tient tout seul, maintenant. Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9918,11 +9916,11 @@
           <t>enfant-m|Papa, tu ouvres le sac ?
 papa|Je l'ouvre, tout doux.
 narrateur|Papa ouvre le sac, tout grand.
-narrateur|Nino glisse un pied, et ses genoux se posent.
+narrateur|Nino glisse un pied, les genoux se posent.
 narrateur|L'autre pied suit, la lampe au calme.
-enfant-m|On demande, et ça va juste.
+enfant-m|Toi tu ouvres, moi j'entre.
 maman|Vous avez demandé, et ça marche.
-papa|Le sac a tenu l'élan.
+papa|Le sac tient tout seul, maintenant.
 narrateur|Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
@@ -9950,12 +9948,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Le sac de papa repose sur le tapis. Tu l'ouvrais, tout grand. On a demandé, et ça allait juste. L'ouverture a fait le tour, rien de plus. Le tapis a rendu le calme. Le sac vert garde un pli chaud, près de la fermeture. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
+          <t>Nino s'allonge, le sac ouvert par papa. Tu l'ouvrais, tout grand. Le sac s'est ouvert, juste assez. L'entrée du camp est à vous. Le tapis a rendu le calme. Le sac vert garde un pli chaud, près de la fermeture. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Le sac de papa repose sur le tapis. Tu l'ouvrais, tout grand. On a demandé, et ça allait juste. L'ouverture a fait le tour, rien de plus. Le tapis a rendu le calme. Le sac vert garde un pli chaud, près de la fermeture. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
+          <t>Nino s'allonge, le sac ouvert par papa. Tu l'ouvrais, tout grand. Le sac s'est ouvert, juste assez. L'entrée du camp est à vous. Le tapis a rendu le calme. Le sac vert garde un pli chaud, près de la fermeture. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10090,10 +10088,10 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|Le sac de papa repose sur le tapis.
+          <t>narrateur|Nino s'allonge, le sac ouvert par papa.
 enfant-m|Tu l'ouvrais, tout grand.
-papa|On a demandé, et ça allait juste.
-maman|L'ouverture a fait le tour, rien de plus.
+papa|Le sac s'est ouvert, juste assez.
+maman|L'entrée du camp est à vous.
 narrateur|Le tapis a rendu le calme.
 narrateur|Le sac vert garde un pli chaud, près de la fermeture.
 narrateur|Un rond de chaleur reste sur le tissu.
@@ -10125,12 +10123,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Le sac vert s'appuie contre le pied du lit. Ici, ça mène au camp, papa. Le bois du lit renvoie chaque pas, tout fort. Nino rebondit, le sac glisse sous le bois. Le sac vert attend au bord, un peu seule. Son élan remplit tout le lit. Toi tu vas plus haut, trop vite. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Nino pousse le sac au pied du lit. Ici, c'est la grotte, papa. Le bois du lit renvoie chaque pas. Le sac se faufile sous le bois, tout seul. Le sac vert n'est plus à sa place. Tes genoux font trop de vagues. Le camp n'a pas encore de toit. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Le sac vert s'appuie contre le pied du lit. Ici, ça mène au camp, papa. Le bois du lit renvoie chaque pas, tout fort. Nino rebondit, le sac glisse sous le bois. Le sac vert attend au bord, un peu seule. Son élan remplit tout le lit. Toi tu vas plus haut, trop vite. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Nino pousse le sac au pied du lit. Ici, c'est la grotte, papa. Le bois du lit renvoie chaque pas. Le sac se faufile sous le bois, tout seul. Le sac vert n'est plus à sa place. Tes genoux font trop de vagues. Le camp n'a pas encore de toit. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10265,13 +10263,13 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Le sac vert s'appuie contre le pied du lit.
-enfant-m|Ici, ça mène au camp, papa.
-narrateur|Le bois du lit renvoie chaque pas, tout fort.
-narrateur|Nino rebondit, le sac glisse sous le bois.
-narrateur|Le sac vert attend au bord, un peu seule.
-maman|Son élan remplit tout le lit.
-papa|Toi tu vas plus haut, trop vite.
+          <t>narrateur|Nino pousse le sac au pied du lit.
+enfant-m|Ici, c'est la grotte, papa.
+narrateur|Le bois du lit renvoie chaque pas.
+narrateur|Le sac se faufile sous le bois, tout seul.
+narrateur|Le sac vert n'est plus à sa place.
+maman|Tes genoux font trop de vagues.
+papa|Le camp n'a pas encore de toit.
 enfant-m|On s'allonge comment, alors ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -10300,12 +10298,12 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore au pied du lit. Les vagues, le matelas, ou maman ?</t>
+          <t>Le bois du lit tremble encore un peu. Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore au pied du lit. Les vagues, le matelas, ou maman ?</t>
+          <t>Le bois du lit tremble encore un peu. Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -10464,7 +10462,7 @@
       <c r="AV53" s="2" t="inlineStr"/>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|Nino rebondit encore au pied du lit.
+          <t>narrateur|Le bois du lit tremble encore un peu.
 papa|Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
@@ -10492,12 +10490,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. Le sac vert voyage d'un genou à l'autre. Ils avancent au pied du lit, l'un après l'autre. Doucement, les vagues tiennent. Vous jouez avec l'élan, ensemble. Le bois est devenu une rive. Le sac vert a fait le tour, sans se taire. Le camp est là, tout bas.</t>
+          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. Le sac voyage d'un genou à l'autre. Le bois devient une mer, puis une rive. Doucement, les vagues tiennent. Vous avez joué, puis calmé le lit. Le pied du lit est une grotte. Le sac vert a trouvé son coin. Le camp est là, tout bas.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. Le sac vert voyage d'un genou à l'autre. Ils avancent au pied du lit, l'un après l'autre. Doucement, les vagues tiennent. Vous jouez avec l'élan, ensemble. Le bois est devenu une rive. Le sac vert a fait le tour, sans se taire. Le camp est là, tout bas.</t>
+          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. Le sac voyage d'un genou à l'autre. Le bois devient une mer, puis une rive. Doucement, les vagues tiennent. Vous avez joué, puis calmé le lit. Le pied du lit est une grotte. Le sac vert a trouvé son coin. Le camp est là, tout bas.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10634,12 +10632,12 @@
         <is>
           <t>enfant-m|On fait des vagues.
 papa|Tu rebondis, puis tu t'arrêtes.
-narrateur|Le sac vert voyage d'un genou à l'autre.
-narrateur|Ils avancent au pied du lit, l'un après l'autre.
+narrateur|Le sac voyage d'un genou à l'autre.
+narrateur|Le bois devient une mer, puis une rive.
 enfant-m|Doucement, les vagues tiennent.
-maman|Vous jouez avec l'élan, ensemble.
-papa|Le bois est devenu une rive.
-narrateur|Le sac vert a fait le tour, sans se taire.
+maman|Vous avez joué, puis calmé le lit.
+papa|Le pied du lit est une grotte.
+narrateur|Le sac vert a trouvé son coin.
 enfant-m|Le camp est là, tout bas.</t>
         </is>
       </c>
@@ -10667,12 +10665,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Les vagues s'arrêtent contre le pied du lit. On est arrivés, tous les deux. Tu rebondissais, puis tu t'arrêtais. Le bois est redevenu un lit, simplement. L'élan s'est couché. Le sac vert garde un pli chaud, près de la fermeture. Une poussière tourne encore, puis tombe. On s'allonge, les vagues se taisent. Dans la chambre, le camp redevient calme.</t>
+          <t>Nino s'allonge au pied du lit. Les vagues sont finies, papa. Tu rebondissais, puis tu t'arrêtais. La grotte a son camp, ce soir. Le bois est redevenu un lit. Le sac vert garde un pli chaud, près de la fermeture. Une poussière tourne encore, puis tombe. Les vagues se taisent. Dans la chambre, le camp tient.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Les vagues s'arrêtent contre le pied du lit. On est arrivés, tous les deux. Tu rebondissais, puis tu t'arrêtais. Le bois est redevenu un lit, simplement. L'élan s'est couché. Le sac vert garde un pli chaud, près de la fermeture. Une poussière tourne encore, puis tombe. On s'allonge, les vagues se taisent. Dans la chambre, le camp redevient calme.</t>
+          <t>Nino s'allonge au pied du lit. Les vagues sont finies, papa. Tu rebondissais, puis tu t'arrêtais. La grotte a son camp, ce soir. Le bois est redevenu un lit. Le sac vert garde un pli chaud, près de la fermeture. Une poussière tourne encore, puis tombe. Les vagues se taisent. Dans la chambre, le camp tient.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10807,15 +10805,15 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|Les vagues s'arrêtent contre le pied du lit.
-enfant-m|On est arrivés, tous les deux.
+          <t>narrateur|Nino s'allonge au pied du lit.
+enfant-m|Les vagues sont finies, papa.
 papa|Tu rebondissais, puis tu t'arrêtais.
-maman|Le bois est redevenu un lit, simplement.
-narrateur|L'élan s'est couché.
+maman|La grotte a son camp, ce soir.
+narrateur|Le bois est redevenu un lit.
 narrateur|Le sac vert garde un pli chaud, près de la fermeture.
 narrateur|Une poussière tourne encore, puis tombe.
-enfant-m|On s'allonge, les vagues se taisent.
-narrateur|Dans la chambre, le camp redevient calme.</t>
+enfant-m|Les vagues se taisent.
+narrateur|Dans la chambre, le camp tient.</t>
         </is>
       </c>
     </row>
@@ -10842,12 +10840,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. Le sac vert reste muet, au creux. Le matelas se tait, enfin. Maintenant ! Vous avez laissé le bois s'ouvrir. L'élan a attendu le pied. Un pli du drap retombe, tout lent.</t>
+          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. Le sac reste fermé, au creux du bois. Le matelas se tait, enfin. Maintenant ! Le lit a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. Le sac vert reste muet, au creux. Le matelas se tait, enfin. Maintenant ! Vous avez laissé le bois s'ouvrir. L'élan a attendu le pied. Un pli du drap retombe, tout lent.</t>
+          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. Le sac reste fermé, au creux du bois. Le matelas se tait, enfin. Maintenant ! Le lit a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -10985,11 +10983,11 @@
           <t>enfant-m|On attend le matelas.
 papa|Quand il se tait, tu t'allonges.
 narrateur|Un saut, puis le bois reste calme.
-narrateur|Le sac vert reste muet, au creux.
+narrateur|Le sac reste fermé, au creux du bois.
 narrateur|Le matelas se tait, enfin.
 enfant-m|Maintenant !
-maman|Vous avez laissé le bois s'ouvrir.
-papa|L'élan a attendu le pied.
+maman|Le lit a fini ses vagues.
+papa|Tes genoux se sont assis, eux aussi.
 narrateur|Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
@@ -11017,12 +11015,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le matelas s'est tu, enfin, tout à fait. On a attendu le bois. Quand il était calme, on s'allongeait. Le pied vous a laissé le sac. L'élan a écouté le bois. Le sac vert ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
+          <t>Nino s'allonge, le matelas tout calme. On a attendu le bois. Quand il s'est tu, tu es entré. Le pied du lit a fait un toit. Tes genoux se sont assis. Le sac vert ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Le matelas s'est tu, enfin, tout à fait. On a attendu le bois. Quand il était calme, on s'allongeait. Le pied vous a laissé le sac. L'élan a écouté le bois. Le sac vert ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
+          <t>Nino s'allonge, le matelas tout calme. On a attendu le bois. Quand il s'est tu, tu es entré. Le pied du lit a fait un toit. Tes genoux se sont assis. Le sac vert ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11157,11 +11155,11 @@
       <c r="AV57" s="2" t="inlineStr"/>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|Le matelas s'est tu, enfin, tout à fait.
+          <t>narrateur|Nino s'allonge, le matelas tout calme.
 enfant-m|On a attendu le bois.
-papa|Quand il était calme, on s'allongeait.
-maman|Le pied vous a laissé le sac.
-narrateur|L'élan a écouté le bois.
+papa|Quand il s'est tu, tu es entré.
+maman|Le pied du lit a fait un toit.
+narrateur|Tes genoux se sont assis.
 narrateur|Le sac vert ne fait plus aucun bruit.
 narrateur|Nino pose la paume sur le bois tiède.
 enfant-m|Il est tiède.
@@ -11192,12 +11190,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac, tout près du bois. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit se range derrière le sac. Vous avez demandé le bord. Mes mains ont tenu l'élan.</t>
+          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac, tout près du bois. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit devient un toit. Vous avez demandé le bord. Mes mains ont tenu le camp.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac, tout près du bois. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit se range derrière le sac. Vous avez demandé le bord. Mes mains ont tenu l'élan.</t>
+          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac, tout près du bois. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit devient un toit. Vous avez demandé le bord. Mes mains ont tenu le camp.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -11338,9 +11336,9 @@
 narrateur|Nino écoute les mains, plus que ses pieds.
 papa|Tu t'allonges, et ça tient.
 enfant-m|Moi aussi, j'écoute.
-narrateur|Le pied du lit se range derrière le sac.
+narrateur|Le pied du lit devient un toit.
 papa|Vous avez demandé le bord.
-maman|Mes mains ont tenu l'élan.</t>
+maman|Mes mains ont tenu le camp.</t>
         </is>
       </c>
     </row>
@@ -11367,12 +11365,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Les mains de maman s'éteignent, un à un. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. Le sac vert garde un pli chaud, près de la fermeture. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
+          <t>Nino s'allonge, le sac bordé par maman. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. Le sac vert garde un pli chaud, près de la fermeture. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Les mains de maman s'éteignent, un à un. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. Le sac vert garde un pli chaud, près de la fermeture. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
+          <t>Nino s'allonge, le sac bordé par maman. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. Le sac vert garde un pli chaud, près de la fermeture. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11507,7 +11505,7 @@
       <c r="AV59" s="2" t="inlineStr"/>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Les mains de maman s'éteignent, un à un.
+          <t>narrateur|Nino s'allonge, le sac bordé par maman.
 enfant-m|J'écoutais tes mains.
 papa|Moi aussi, je bordais avec toi.
 maman|Vous avez demandé le bord.
@@ -11902,12 +11900,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Contre le ventre. Oui. L'oreiller rayé avance, un pas après l'autre. Le départ du camp est là. Les chaussettes de Nino s'arrêtent trop haut. Les talons restent libres, trop vifs. La chambre est tiède, devant. On y va, tous les trois ? Oui.</t>
+          <t>Contre le ventre. Oui. Les rayures de l'oreiller dansent un peu. Ma tête campe dessus. Nino le serre, le lâche, le reprend. Un coin rayé frotte sa joue, tout doux. La chambre est prête, devant. On y va, tous les trois ? Oui.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Contre le ventre. Oui. L'oreiller rayé avance, un pas après l'autre. Le départ du camp est là. Les chaussettes de Nino s'arrêtent trop haut. Les talons restent libres, trop vifs. La chambre est tiède, devant. On y va, tous les trois ? Oui.</t>
+          <t>Contre le ventre. Oui. Les rayures de l'oreiller dansent un peu. Ma tête campe dessus. Nino le serre, le lâche, le reprend. Un coin rayé frotte sa joue, tout doux. La chambre est prête, devant. On y va, tous les trois ? Oui.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -12048,11 +12046,11 @@
         <is>
           <t>enfant-m|Contre le ventre.
 maman|Oui.
-narrateur|L'oreiller rayé avance, un pas après l'autre.
-enfant-m|Le départ du camp est là.
-narrateur|Les chaussettes de Nino s'arrêtent trop haut.
-narrateur|Les talons restent libres, trop vifs.
-maman|La chambre est tiède, devant.
+narrateur|Les rayures de l'oreiller dansent un peu.
+enfant-m|Ma tête campe dessus.
+narrateur|Nino le serre, le lâche, le reprend.
+narrateur|Un coin rayé frotte sa joue, tout doux.
+maman|La chambre est prête, devant.
 papa|On y va, tous les trois ?
 enfant-m|Oui.</t>
         </is>
@@ -12081,12 +12079,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Nino tapote déjà le parquet, tout léger. La fenêtre garde un rai de rue. Le tapis fait un carré chaud. Le pied du lit attend, tout bas. On campe où, Nino ?</t>
+          <t>Nino tapote déjà le parquet, tout léger. Sous la fenêtre, le rideau garde un rai de rue. Au milieu, le tapis fait un carré chaud. Près du bois, le pied du lit attend. On campe où, Nino ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Nino tapote déjà le parquet, tout léger. La fenêtre garde un rai de rue. Le tapis fait un carré chaud. Le pied du lit attend, tout bas. On campe où, Nino ?</t>
+          <t>Nino tapote déjà le parquet, tout léger. Sous la fenêtre, le rideau garde un rai de rue. Au milieu, le tapis fait un carré chaud. Près du bois, le pied du lit attend. On campe où, Nino ?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -12246,9 +12244,9 @@
       <c r="AW63" t="inlineStr">
         <is>
           <t>narrateur|Nino tapote déjà le parquet, tout léger.
-narrateur|La fenêtre garde un rai de rue.
-narrateur|Le tapis fait un carré chaud.
-narrateur|Le pied du lit attend, tout bas.
+narrateur|Sous la fenêtre, le rideau garde un rai de rue.
+narrateur|Au milieu, le tapis fait un carré chaud.
+narrateur|Près du bois, le pied du lit attend.
 papa|On campe où, Nino ?</t>
         </is>
       </c>
@@ -12276,12 +12274,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>L'oreiller rayé avance vers la fenêtre. Nino tape le parquet, trop vite. Moi je cours, papa ! Ses pieds font des ronds, trop larges. L'oreiller heurte le rebord, puis rebondit. L'oreiller rayé n'attendait pas ça. Il a envie de bouger, c'est tout. Tes jambes sont plus vives, ce soir. On campe comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Nino pousse l'oreiller vers le rideau. Ses talons tambourinent le parquet. Le camp, c'est là, papa ! L'oreiller tape le bois, rebondit trop haut. L'oreiller rayé part trop vite. Tes pieds dansent, ce soir. Le rideau n'est pas encore une tente. On campe comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>L'oreiller rayé avance vers la fenêtre. Nino tape le parquet, trop vite. Moi je cours, papa ! Ses pieds font des ronds, trop larges. L'oreiller heurte le rebord, puis rebondit. L'oreiller rayé n'attendait pas ça. Il a envie de bouger, c'est tout. Tes jambes sont plus vives, ce soir. On campe comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Nino pousse l'oreiller vers le rideau. Ses talons tambourinent le parquet. Le camp, c'est là, papa ! L'oreiller tape le bois, rebondit trop haut. L'oreiller rayé part trop vite. Tes pieds dansent, ce soir. Le rideau n'est pas encore une tente. On campe comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12416,14 +12414,13 @@
       <c r="AV64" s="2" t="inlineStr"/>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>narrateur|L'oreiller rayé avance vers la fenêtre.
-narrateur|Nino tape le parquet, trop vite.
-enfant-m|Moi je cours, papa !
-narrateur|Ses pieds font des ronds, trop larges.
-narrateur|L'oreiller heurte le rebord, puis rebondit.
-enfant-m|L'oreiller rayé n'attendait pas ça.
-maman|Il a envie de bouger, c'est tout.
-papa|Tes jambes sont plus vives, ce soir.
+          <t>narrateur|Nino pousse l'oreiller vers le rideau.
+narrateur|Ses talons tambourinent le parquet.
+enfant-m|Le camp, c'est là, papa !
+narrateur|L'oreiller tape le bois, rebondit trop haut.
+enfant-m|L'oreiller rayé part trop vite.
+maman|Tes pieds dansent, ce soir.
+papa|Le rideau n'est pas encore une tente.
 enfant-m|On campe comment, alors ?
 papa|Tu fais comment, avec nous ?</t>
         </is>
@@ -12452,12 +12449,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Nino tape encore le parquet, tout fort. Les lucioles, le rideau, ou maman ?</t>
+          <t>Le lapin de lumière court encore. Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Nino tape encore le parquet, tout fort. Les lucioles, le rideau, ou maman ?</t>
+          <t>Le lapin de lumière court encore. Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -12616,7 +12613,7 @@
       <c r="AV65" s="2" t="inlineStr"/>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|Nino tape encore le parquet, tout fort.
+          <t>narrateur|Le lapin de lumière court encore.
 papa|Les lucioles, le rideau, ou maman ?</t>
         </is>
       </c>
@@ -12644,12 +12641,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>On joue aux lucioles. Toi tu bouges, moi je suis le rond. Nino tient l'oreiller, le faisceau danse. Deux ronds se croisent sur le rideau. Nino saute une fois, puis s'arrête. Maintenant c'est le camp. L'élan a trouvé sa fenêtre. Vous jouez à tour, sur le tissu. Le rideau redevient un mur, tout doux.</t>
+          <t>On joue aux lucioles. Toi tu clignes, moi je compte. Nino cligne, l'oreiller devient un nuage. Des points d'or s'allument sur le rideau. Nino cligne encore, puis s'arrête. Les lucioles sont fatiguées. Le camp a sa lumière, maintenant. Vous avez dansé, puis posé. Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>On joue aux lucioles. Toi tu bouges, moi je suis le rond. Nino tient l'oreiller, le faisceau danse. Deux ronds se croisent sur le rideau. Nino saute une fois, puis s'arrête. Maintenant c'est le camp. L'élan a trouvé sa fenêtre. Vous jouez à tour, sur le tissu. Le rideau redevient un mur, tout doux.</t>
+          <t>On joue aux lucioles. Toi tu clignes, moi je compte. Nino cligne, l'oreiller devient un nuage. Des points d'or s'allument sur le rideau. Nino cligne encore, puis s'arrête. Les lucioles sont fatiguées. Le camp a sa lumière, maintenant. Vous avez dansé, puis posé. Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12785,14 +12782,14 @@
       <c r="AW66" t="inlineStr">
         <is>
           <t>enfant-m|On joue aux lucioles.
-papa|Toi tu bouges, moi je suis le rond.
-narrateur|Nino tient l'oreiller, le faisceau danse.
-narrateur|Deux ronds se croisent sur le rideau.
-narrateur|Nino saute une fois, puis s'arrête.
-enfant-m|Maintenant c'est le camp.
-maman|L'élan a trouvé sa fenêtre.
-papa|Vous jouez à tour, sur le tissu.
-narrateur|Le rideau redevient un mur, tout doux.</t>
+papa|Toi tu clignes, moi je compte.
+narrateur|Nino cligne, l'oreiller devient un nuage.
+narrateur|Des points d'or s'allument sur le rideau.
+narrateur|Nino cligne encore, puis s'arrête.
+enfant-m|Les lucioles sont fatiguées.
+maman|Le camp a sa lumière, maintenant.
+papa|Vous avez dansé, puis posé.
+narrateur|Le tissu redevient un mur, tout doux.</t>
         </is>
       </c>
     </row>
@@ -12819,12 +12816,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le dernier rond du rideau est à eux. On a joué, chacun son tour. Toi tu bougais, moi je suivais. Vous avez laissé l'élan dessiner. La chambre sent encore le savon. L'oreiller rayé garde une chaleur ronde, au creux. Un trait clair dort sur le bois. On s'allonge, papa. Les chaussettes retrouvent le tapis tiède.</t>
+          <t>Nino s'allonge, le sac sous le rideau. Les lucioles sont couchées, papa. Toi tu clignais, moi je comptais. Le camp a sa lumière, ce soir. La chambre sent encore le savon. L'oreiller rayé garde une chaleur ronde, au creux. Un point d'or dort sur le tissu. Bonne nuit, fenêtre. Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Le dernier rond du rideau est à eux. On a joué, chacun son tour. Toi tu bougais, moi je suivais. Vous avez laissé l'élan dessiner. La chambre sent encore le savon. L'oreiller rayé garde une chaleur ronde, au creux. Un trait clair dort sur le bois. On s'allonge, papa. Les chaussettes retrouvent le tapis tiède.</t>
+          <t>Nino s'allonge, le sac sous le rideau. Les lucioles sont couchées, papa. Toi tu clignais, moi je comptais. Le camp a sa lumière, ce soir. La chambre sent encore le savon. L'oreiller rayé garde une chaleur ronde, au creux. Un point d'or dort sur le tissu. Bonne nuit, fenêtre. Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12959,14 +12956,14 @@
       <c r="AV67" s="2" t="inlineStr"/>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|Le dernier rond du rideau est à eux.
-enfant-m|On a joué, chacun son tour.
-papa|Toi tu bougais, moi je suivais.
-maman|Vous avez laissé l'élan dessiner.
+          <t>narrateur|Nino s'allonge, le sac sous le rideau.
+enfant-m|Les lucioles sont couchées, papa.
+papa|Toi tu clignais, moi je comptais.
+maman|Le camp a sa lumière, ce soir.
 narrateur|La chambre sent encore le savon.
 narrateur|L'oreiller rayé garde une chaleur ronde, au creux.
-narrateur|Un trait clair dort sur le bois.
-enfant-m|On s'allonge, papa.
+narrateur|Un point d'or dort sur le tissu.
+enfant-m|Bonne nuit, fenêtre.
 narrateur|Les chaussettes retrouvent le tapis tiède.</t>
         </is>
       </c>
@@ -12994,12 +12991,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu. Nino pose les genoux au bois. L'oreiller rayé attend près du rebord. Sa respiration redevient calme, tout doux. Je suis prêt ? Le rideau ne bouge plus. Vous avez laissé l'élan s'asseoir. Le faisceau tient enfin, tout droit. Le camp peut s'ouvrir.</t>
+          <t>On attend le rideau. Nino pose les genoux au parquet. L'oreiller repose contre le rebord, sage. Le volet tape une fois, puis plus. Il ne bouge plus ? Le tissu est calme, oui. Tes pieds se sont assis, eux aussi. Nino rallume, tout droit, tout petit. Le camp peut s'ouvrir.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu. Nino pose les genoux au bois. L'oreiller rayé attend près du rebord. Sa respiration redevient calme, tout doux. Je suis prêt ? Le rideau ne bouge plus. Vous avez laissé l'élan s'asseoir. Le faisceau tient enfin, tout droit. Le camp peut s'ouvrir.</t>
+          <t>On attend le rideau. Nino pose les genoux au parquet. L'oreiller repose contre le rebord, sage. Le volet tape une fois, puis plus. Il ne bouge plus ? Le tissu est calme, oui. Tes pieds se sont assis, eux aussi. Nino rallume, tout droit, tout petit. Le camp peut s'ouvrir.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13134,14 +13131,14 @@
       <c r="AV68" s="2" t="inlineStr"/>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>enfant-m|On attend un peu.
-narrateur|Nino pose les genoux au bois.
-narrateur|L'oreiller rayé attend près du rebord.
-narrateur|Sa respiration redevient calme, tout doux.
-enfant-m|Je suis prêt ?
-maman|Le rideau ne bouge plus.
-papa|Vous avez laissé l'élan s'asseoir.
-narrateur|Le faisceau tient enfin, tout droit.
+          <t>enfant-m|On attend le rideau.
+narrateur|Nino pose les genoux au parquet.
+narrateur|L'oreiller repose contre le rebord, sage.
+narrateur|Le volet tape une fois, puis plus.
+enfant-m|Il ne bouge plus ?
+maman|Le tissu est calme, oui.
+papa|Tes pieds se sont assis, eux aussi.
+narrateur|Nino rallume, tout droit, tout petit.
 enfant-m|Le camp peut s'ouvrir.</t>
         </is>
       </c>
@@ -13169,12 +13166,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le rebord de la fenêtre garde encore la chaleur. Je me suis arrêté, d'abord. Puis le faisceau est resté droit. L'élan s'est assis, puis il a campé. Le rideau redevient calme. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
+          <t>Nino s'allonge, le rideau tout calme. J'ai attendu le volet, d'abord. Puis le faisceau est resté droit. Tes pieds se sont assis, eux aussi. Le tissu ne danse plus. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Le rebord de la fenêtre garde encore la chaleur. Je me suis arrêté, d'abord. Puis le faisceau est resté droit. L'élan s'est assis, puis il a campé. Le rideau redevient calme. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
+          <t>Nino s'allonge, le rideau tout calme. J'ai attendu le volet, d'abord. Puis le faisceau est resté droit. Tes pieds se sont assis, eux aussi. Le tissu ne danse plus. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière reste coincée, tout près. À demain, les ronds. Le volet brille un peu, puis se tait.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13309,11 +13306,11 @@
       <c r="AV69" s="2" t="inlineStr"/>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|Le rebord de la fenêtre garde encore la chaleur.
-enfant-m|Je me suis arrêté, d'abord.
+          <t>narrateur|Nino s'allonge, le rideau tout calme.
+enfant-m|J'ai attendu le volet, d'abord.
 papa|Puis le faisceau est resté droit.
-maman|L'élan s'est assis, puis il a campé.
-narrateur|Le rideau redevient calme.
+maman|Tes pieds se sont assis, eux aussi.
+narrateur|Le tissu ne danse plus.
 narrateur|L'oreiller rayé garde une chaleur ronde, au creux.
 narrateur|Une poussière reste coincée, tout près.
 enfant-m|À demain, les ronds.
@@ -13344,12 +13341,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens la lampe ? Je la tiens, un pas chacun. Maman pose l'oreiller près de sa main. Nino pose un pied, puis l'autre. Le faisceau reste sage, juste à côté. On demande, et ça va ! Vous avez demandé, tout calme. Ma main a juste attendu. La fenêtre garde un rai, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu poses le camp. Maman tient l'oreiller, Nino tend la lampe. Nino étale le sac sous le rai de rue. Le faisceau reste sage, dans sa main. Toi tu tiens, moi je range. Vous avez demandé, et ça tient. Ma main fait le piquet, ce soir. La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens la lampe ? Je la tiens, un pas chacun. Maman pose l'oreiller près de sa main. Nino pose un pied, puis l'autre. Le faisceau reste sage, juste à côté. On demande, et ça va ! Vous avez demandé, tout calme. Ma main a juste attendu. La fenêtre garde un rai, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu poses le camp. Maman tient l'oreiller, Nino tend la lampe. Nino étale le sac sous le rai de rue. Le faisceau reste sage, dans sa main. Toi tu tiens, moi je range. Vous avez demandé, et ça tient. Ma main fait le piquet, ce soir. La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13484,14 +13481,14 @@
       <c r="AV70" s="2" t="inlineStr"/>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>enfant-m|Maman, tu tiens la lampe ?
-maman|Je la tiens, un pas chacun.
-narrateur|Maman pose l'oreiller près de sa main.
-narrateur|Nino pose un pied, puis l'autre.
-narrateur|Le faisceau reste sage, juste à côté.
-enfant-m|On demande, et ça va !
-papa|Vous avez demandé, tout calme.
-maman|Ma main a juste attendu.
+          <t>enfant-m|Maman, tu tiens, s'il te plaît ?
+maman|Je tiens, tu poses le camp.
+narrateur|Maman tient l'oreiller, Nino tend la lampe.
+narrateur|Nino étale le sac sous le rai de rue.
+narrateur|Le faisceau reste sage, dans sa main.
+enfant-m|Toi tu tiens, moi je range.
+papa|Vous avez demandé, et ça tient.
+maman|Ma main fait le piquet, ce soir.
 narrateur|La fenêtre garde un rai, tout mince.</t>
         </is>
       </c>
@@ -13519,12 +13516,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>La main de maman reste dans l'air, tout légère. J'ai attendu le pas. On a demandé, et ça allait. Sa main a tenu vos pieds. La chambre vous rend le silence. L'oreiller rayé pose un grain de lumière sur le bois. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
+          <t>Nino s'allonge, la main de maman tout près. Tu tenais le piquet. Vous avez demandé, et ça tenait. Ma main a fait la tente. La chambre rend le silence, tout doux. L'oreiller rayé pose un grain de lumière. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>La main de maman reste dans l'air, tout légère. J'ai attendu le pas. On a demandé, et ça allait. Sa main a tenu vos pieds. La chambre vous rend le silence. L'oreiller rayé pose un grain de lumière sur le bois. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
+          <t>Nino s'allonge, la main de maman tout près. Tu tenais le piquet. Vous avez demandé, et ça tenait. Ma main a fait la tente. La chambre rend le silence, tout doux. L'oreiller rayé pose un grain de lumière. Nino touche le rideau, du bout. Il est à nous. Un rai de rue barre encore le tissu.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13659,12 +13656,12 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|La main de maman reste dans l'air, tout légère.
-enfant-m|J'ai attendu le pas.
-papa|On a demandé, et ça allait.
-maman|Sa main a tenu vos pieds.
-narrateur|La chambre vous rend le silence.
-narrateur|L'oreiller rayé pose un grain de lumière sur le bois.
+          <t>narrateur|Nino s'allonge, la main de maman tout près.
+enfant-m|Tu tenais le piquet.
+papa|Vous avez demandé, et ça tenait.
+maman|Ma main a fait la tente.
+narrateur|La chambre rend le silence, tout doux.
+narrateur|L'oreiller rayé pose un grain de lumière.
 narrateur|Nino touche le rideau, du bout.
 enfant-m|Il est à nous.
 narrateur|Un rai de rue barre encore le tissu.</t>
@@ -13694,12 +13691,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>L'oreiller rayé bute au milieu du tapis. Le tapis est à nous, maman. Ses pieds quittent le tissu, puis reviennent. Nino saute par-dessus l'oreiller, sans s'arrêter. Un peu de poussière lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, trop vite. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Nino jette l'oreiller au milieu du tapis. Ici, c'est la clairière, maman. Ses genoux font un petit trampoline. L'oreiller file, une rayure après l'autre. Un fil de laine se lève, puis retombe. Ton corps veut encore courir. Le tapis n'a pas encore de tente. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>L'oreiller rayé bute au milieu du tapis. Le tapis est à nous, maman. Ses pieds quittent le tissu, puis reviennent. Nino saute par-dessus l'oreiller, sans s'arrêter. Un peu de poussière lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, trop vite. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Nino jette l'oreiller au milieu du tapis. Ici, c'est la clairière, maman. Ses genoux font un petit trampoline. L'oreiller file, une rayure après l'autre. Un fil de laine se lève, puis retombe. Ton corps veut encore courir. Le tapis n'a pas encore de tente. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13834,13 +13831,13 @@
       <c r="AV72" s="2" t="inlineStr"/>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>narrateur|L'oreiller rayé bute au milieu du tapis.
-enfant-m|Le tapis est à nous, maman.
-narrateur|Ses pieds quittent le tissu, puis reviennent.
-narrateur|Nino saute par-dessus l'oreiller, sans s'arrêter.
-narrateur|Un peu de poussière lève, puis retombe.
-maman|Il a de l'élan, comme un petit vent.
-papa|Toi tu vas plus loin, trop vite.
+          <t>narrateur|Nino jette l'oreiller au milieu du tapis.
+enfant-m|Ici, c'est la clairière, maman.
+narrateur|Ses genoux font un petit trampoline.
+narrateur|L'oreiller file, une rayure après l'autre.
+narrateur|Un fil de laine se lève, puis retombe.
+maman|Ton corps veut encore courir.
+papa|Le tapis n'a pas encore de tente.
 enfant-m|On peut jouer avec, quand même ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -13869,12 +13866,12 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore sur le tapis. Le sentier, la fermeture, ou papa ?</t>
+          <t>Le sac n'a pas encore de forme. Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore sur le tapis. Le sentier, la fermeture, ou papa ?</t>
+          <t>Le sac n'a pas encore de forme. Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -14033,7 +14030,7 @@
       <c r="AV73" s="2" t="inlineStr"/>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|Nino rebondit encore sur le tapis.
+          <t>narrateur|Le sac n'a pas encore de forme.
 maman|Le sentier, la fermeture, ou papa ?</t>
         </is>
       </c>
@@ -14061,12 +14058,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On fait un sentier. Toi derrière, moi devant ! Nino garde l'oreiller, papa saute devant. Deux ombres passent sur le même tapis. Nino va plus vite, papa plus loin. On arrive au bout, tous les deux. Vous avez joué avec l'élan. Le tapis vous a laissés passer. Un fil de laine reste, tout petit.</t>
+          <t>On fait un sentier. Toi tu sautes, moi je suis derrière. Nino pose l'oreiller, papa marque le sentier. Des pas dessinent un chemin sur le tapis. Nino saute une case, papa une autre. La clairière est au bout. Vous avez joué, puis posé le sac. Le tapis est devenu un chemin. Un fil de laine reste, tout petit.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>On fait un sentier. Toi derrière, moi devant ! Nino garde l'oreiller, papa saute devant. Deux ombres passent sur le même tapis. Nino va plus vite, papa plus loin. On arrive au bout, tous les deux. Vous avez joué avec l'élan. Le tapis vous a laissés passer. Un fil de laine reste, tout petit.</t>
+          <t>On fait un sentier. Toi tu sautes, moi je suis derrière. Nino pose l'oreiller, papa marque le sentier. Des pas dessinent un chemin sur le tapis. Nino saute une case, papa une autre. La clairière est au bout. Vous avez joué, puis posé le sac. Le tapis est devenu un chemin. Un fil de laine reste, tout petit.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14202,13 +14199,13 @@
       <c r="AW74" t="inlineStr">
         <is>
           <t>enfant-m|On fait un sentier.
-papa|Toi derrière, moi devant !
-narrateur|Nino garde l'oreiller, papa saute devant.
-narrateur|Deux ombres passent sur le même tapis.
-narrateur|Nino va plus vite, papa plus loin.
-enfant-m|On arrive au bout, tous les deux.
-maman|Vous avez joué avec l'élan.
-papa|Le tapis vous a laissés passer.
+papa|Toi tu sautes, moi je suis derrière.
+narrateur|Nino pose l'oreiller, papa marque le sentier.
+narrateur|Des pas dessinent un chemin sur le tapis.
+narrateur|Nino saute une case, papa une autre.
+enfant-m|La clairière est au bout.
+maman|Vous avez joué, puis posé le sac.
+papa|Le tapis est devenu un chemin.
 narrateur|Un fil de laine reste, tout petit.</t>
         </is>
       </c>
@@ -14236,12 +14233,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Deux paires de chaussettes marquent le bout du tapis. Toi devant, moi derrière. Tes jambes allaient plus loin. Vous avez sauté avec l'élan, pas contre. Le tapis redevient chaud, et calme. L'oreiller rayé garde une chaleur ronde, au creux. Un peu de laine sèche déjà sur le tissu. On s'allonge, le sentier reste. Le lit fait une ombre longue.</t>
+          <t>Nino s'allonge au bout du sentier. Toi devant, moi derrière. Tes sauts ont fait le chemin. La clairière est devenue un camp. Le tapis redevient chaud, et calme. L'oreiller rayé garde une chaleur ronde, au creux. Un peu de laine sèche déjà. Le sentier reste, maman. Le lit fait une ombre longue.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Deux paires de chaussettes marquent le bout du tapis. Toi devant, moi derrière. Tes jambes allaient plus loin. Vous avez sauté avec l'élan, pas contre. Le tapis redevient chaud, et calme. L'oreiller rayé garde une chaleur ronde, au creux. Un peu de laine sèche déjà sur le tissu. On s'allonge, le sentier reste. Le lit fait une ombre longue.</t>
+          <t>Nino s'allonge au bout du sentier. Toi devant, moi derrière. Tes sauts ont fait le chemin. La clairière est devenue un camp. Le tapis redevient chaud, et calme. L'oreiller rayé garde une chaleur ronde, au creux. Un peu de laine sèche déjà. Le sentier reste, maman. Le lit fait une ombre longue.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14376,14 +14373,14 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|Deux paires de chaussettes marquent le bout du tapis.
+          <t>narrateur|Nino s'allonge au bout du sentier.
 enfant-m|Toi devant, moi derrière.
-papa|Tes jambes allaient plus loin.
-maman|Vous avez sauté avec l'élan, pas contre.
+papa|Tes sauts ont fait le chemin.
+maman|La clairière est devenue un camp.
 narrateur|Le tapis redevient chaud, et calme.
 narrateur|L'oreiller rayé garde une chaleur ronde, au creux.
-narrateur|Un peu de laine sèche déjà sur le tissu.
-enfant-m|On s'allonge, le sentier reste.
+narrateur|Un peu de laine sèche déjà.
+enfant-m|Le sentier reste, maman.
 narrateur|Le lit fait une ombre longue.</t>
         </is>
       </c>
@@ -14411,12 +14408,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient l'oreiller, sur le tissu. La fermeture avance, tout seule d'abord. Nino souffle, puis il recule. C'est à toi, Nino. Merci, j'y vais. Chacun son tour, sur le tapis. L'élan a attendu la place.</t>
+          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient l'oreiller, le sac attend. Le zip avance, dent après dent. Nino souffle, les épaules baissent. C'est à toi, Nino. J'y glisse un pied. Chacun son tour, sur le tapis. La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient l'oreiller, sur le tissu. La fermeture avance, tout seule d'abord. Nino souffle, puis il recule. C'est à toi, Nino. Merci, j'y vais. Chacun son tour, sur le tapis. L'élan a attendu la place.</t>
+          <t>J'attends la fermeture. Moi je l'ouvre, puis c'est toi. Nino tient l'oreiller, le sac attend. Le zip avance, dent après dent. Nino souffle, les épaules baissent. C'est à toi, Nino. J'y glisse un pied. Chacun son tour, sur le tapis. La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14553,13 +14550,13 @@
         <is>
           <t>enfant-m|J'attends la fermeture.
 papa|Moi je l'ouvre, puis c'est toi.
-narrateur|Nino tient l'oreiller, sur le tissu.
-narrateur|La fermeture avance, tout seule d'abord.
-narrateur|Nino souffle, puis il recule.
+narrateur|Nino tient l'oreiller, le sac attend.
+narrateur|Le zip avance, dent après dent.
+narrateur|Nino souffle, les épaules baissent.
 papa|C'est à toi, Nino.
-enfant-m|Merci, j'y vais.
+enfant-m|J'y glisse un pied.
 maman|Chacun son tour, sur le tapis.
-narrateur|L'élan a attendu la place.</t>
+narrateur|La tente verte s'ouvre, enfin.</t>
         </is>
       </c>
     </row>
@@ -14586,12 +14583,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le bout du tapis attend encore, tout lisse. J'ai ouvert, puis c'était toi. J'ai attendu ta place. Chacun son tour, sur le tissu. L'élan a laissé la place. L'oreiller rayé garde un grain de poussière. Nino souffle dessus, tout doux. On se dit au revoir, tapis. Un fil oublié sèche contre le pied.</t>
+          <t>Nino s'allonge dans le sac ouvert. J'ai ouvert, puis c'était toi. J'ai attendu le zip. Chacun son tour, sur le tapis. La tente verte tient, enfin. L'oreiller rayé garde un grain de poussière. Nino souffle dessus, tout doux. Bonne nuit, tapis. Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Le bout du tapis attend encore, tout lisse. J'ai ouvert, puis c'était toi. J'ai attendu ta place. Chacun son tour, sur le tissu. L'élan a laissé la place. L'oreiller rayé garde un grain de poussière. Nino souffle dessus, tout doux. On se dit au revoir, tapis. Un fil oublié sèche contre le pied.</t>
+          <t>Nino s'allonge dans le sac ouvert. J'ai ouvert, puis c'était toi. J'ai attendu le zip. Chacun son tour, sur le tapis. La tente verte tient, enfin. L'oreiller rayé garde un grain de poussière. Nino souffle dessus, tout doux. Bonne nuit, tapis. Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14726,14 +14723,14 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Le bout du tapis attend encore, tout lisse.
+          <t>narrateur|Nino s'allonge dans le sac ouvert.
 papa|J'ai ouvert, puis c'était toi.
-enfant-m|J'ai attendu ta place.
-maman|Chacun son tour, sur le tissu.
-narrateur|L'élan a laissé la place.
+enfant-m|J'ai attendu le zip.
+maman|Chacun son tour, sur le tapis.
+narrateur|La tente verte tient, enfin.
 narrateur|L'oreiller rayé garde un grain de poussière.
 narrateur|Nino souffle dessus, tout doux.
-enfant-m|On se dit au revoir, tapis.
+enfant-m|Bonne nuit, tapis.
 narrateur|Un fil oublié sèche contre le pied.</t>
         </is>
       </c>
@@ -14761,12 +14758,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de l'oreiller. Nino glisse un pied, et ses genoux se posent. L'autre pied suit, la lampe au calme. On demande, et ça va juste. Vous avez demandé, et ça marche. Le sac a tenu l'élan. Un carré de tapis reste tiède, autour.</t>
+          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de l'oreiller. Nino glisse un pied, les genoux se posent. L'autre pied suit, la lampe au calme. Toi tu ouvres, moi j'entre. Vous avez demandé, et ça marche. Le sac tient tout seul, maintenant. Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de l'oreiller. Nino glisse un pied, et ses genoux se posent. L'autre pied suit, la lampe au calme. On demande, et ça va juste. Vous avez demandé, et ça marche. Le sac a tenu l'élan. Un carré de tapis reste tiède, autour.</t>
+          <t>Papa, tu ouvres le sac ? Je l'ouvre, tout doux. Papa ouvre le sac près de l'oreiller. Nino glisse un pied, les genoux se posent. L'autre pied suit, la lampe au calme. Toi tu ouvres, moi j'entre. Vous avez demandé, et ça marche. Le sac tient tout seul, maintenant. Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14904,11 +14901,11 @@
           <t>enfant-m|Papa, tu ouvres le sac ?
 papa|Je l'ouvre, tout doux.
 narrateur|Papa ouvre le sac près de l'oreiller.
-narrateur|Nino glisse un pied, et ses genoux se posent.
+narrateur|Nino glisse un pied, les genoux se posent.
 narrateur|L'autre pied suit, la lampe au calme.
-enfant-m|On demande, et ça va juste.
+enfant-m|Toi tu ouvres, moi j'entre.
 maman|Vous avez demandé, et ça marche.
-papa|Le sac a tenu l'élan.
+papa|Le sac tient tout seul, maintenant.
 narrateur|Un carré de tapis reste tiède, autour.</t>
         </is>
       </c>
@@ -14936,12 +14933,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Le sac de papa repose sur le tapis. Tu l'ouvrais, tout grand. On a demandé, et ça allait juste. L'ouverture a fait le tour, rien de plus. Le tapis a rendu le calme. L'oreiller rayé garde une chaleur ronde, au creux. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
+          <t>Nino s'allonge, le sac ouvert par papa. Tu l'ouvrais, tout grand. Le sac s'est ouvert, juste assez. L'entrée du camp est à vous. Le tapis a rendu le calme. L'oreiller rayé garde une chaleur ronde, au creux. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Le sac de papa repose sur le tapis. Tu l'ouvrais, tout grand. On a demandé, et ça allait juste. L'ouverture a fait le tour, rien de plus. Le tapis a rendu le calme. L'oreiller rayé garde une chaleur ronde, au creux. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
+          <t>Nino s'allonge, le sac ouvert par papa. Tu l'ouvrais, tout grand. Le sac s'est ouvert, juste assez. L'entrée du camp est à vous. Le tapis a rendu le calme. L'oreiller rayé garde une chaleur ronde, au creux. Un rond de chaleur reste sur le tissu. Regarde, papa, il brille. Les chaussettes retrouvent le parquet, au frais.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15076,10 +15073,10 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|Le sac de papa repose sur le tapis.
+          <t>narrateur|Nino s'allonge, le sac ouvert par papa.
 enfant-m|Tu l'ouvrais, tout grand.
-papa|On a demandé, et ça allait juste.
-maman|L'ouverture a fait le tour, rien de plus.
+papa|Le sac s'est ouvert, juste assez.
+maman|L'entrée du camp est à vous.
 narrateur|Le tapis a rendu le calme.
 narrateur|L'oreiller rayé garde une chaleur ronde, au creux.
 narrateur|Un rond de chaleur reste sur le tissu.
@@ -15111,12 +15108,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>L'oreiller rayé s'arrête près du pied du lit. Ici, ça mène au camp, papa. Le bois du lit renvoie chaque pas, tout fort. Nino rebondit, l'oreiller file sous le drap. L'oreiller rayé attend au bord, un peu seule. Son élan remplit tout le lit. Toi tu vas plus haut, trop vite. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Nino pose l'oreiller au pied du lit. Ici, c'est la grotte, papa. Le bois du lit renvoie chaque pas. L'oreiller disparaît sous le drap, trop loin. L'oreiller rayé n'est plus à sa place. Tes genoux font trop de vagues. Le camp n'a pas encore de toit. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>L'oreiller rayé s'arrête près du pied du lit. Ici, ça mène au camp, papa. Le bois du lit renvoie chaque pas, tout fort. Nino rebondit, l'oreiller file sous le drap. L'oreiller rayé attend au bord, un peu seule. Son élan remplit tout le lit. Toi tu vas plus haut, trop vite. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Nino pose l'oreiller au pied du lit. Ici, c'est la grotte, papa. Le bois du lit renvoie chaque pas. L'oreiller disparaît sous le drap, trop loin. L'oreiller rayé n'est plus à sa place. Tes genoux font trop de vagues. Le camp n'a pas encore de toit. On s'allonge comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15251,13 +15248,13 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|L'oreiller rayé s'arrête près du pied du lit.
-enfant-m|Ici, ça mène au camp, papa.
-narrateur|Le bois du lit renvoie chaque pas, tout fort.
-narrateur|Nino rebondit, l'oreiller file sous le drap.
-narrateur|L'oreiller rayé attend au bord, un peu seule.
-maman|Son élan remplit tout le lit.
-papa|Toi tu vas plus haut, trop vite.
+          <t>narrateur|Nino pose l'oreiller au pied du lit.
+enfant-m|Ici, c'est la grotte, papa.
+narrateur|Le bois du lit renvoie chaque pas.
+narrateur|L'oreiller disparaît sous le drap, trop loin.
+narrateur|L'oreiller rayé n'est plus à sa place.
+maman|Tes genoux font trop de vagues.
+papa|Le camp n'a pas encore de toit.
 enfant-m|On s'allonge comment, alors ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -15286,12 +15283,12 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore au pied du lit. Les vagues, le matelas, ou maman ?</t>
+          <t>Le bois du lit tremble encore un peu. Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Nino rebondit encore au pied du lit. Les vagues, le matelas, ou maman ?</t>
+          <t>Le bois du lit tremble encore un peu. Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -15450,7 +15447,7 @@
       <c r="AV81" s="2" t="inlineStr"/>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|Nino rebondit encore au pied du lit.
+          <t>narrateur|Le bois du lit tremble encore un peu.
 papa|Les vagues, le matelas, ou maman ?</t>
         </is>
       </c>
@@ -15478,12 +15475,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. L'oreiller rayé voyage d'un genou à l'autre. Ils avancent au pied du lit, l'un après l'autre. Doucement, les vagues tiennent. Vous jouez avec l'élan, ensemble. Le bois est devenu une rive. L'oreiller rayé a fait le tour, sans se taire. Le camp est là, tout bas.</t>
+          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. L'oreiller voyage d'un genou à l'autre. Le bois devient une mer, puis une rive. Doucement, les vagues tiennent. Vous avez joué, puis calmé le lit. Le pied du lit est une grotte. L'oreiller rayé a trouvé son coin. Le camp est là, tout bas.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. L'oreiller rayé voyage d'un genou à l'autre. Ils avancent au pied du lit, l'un après l'autre. Doucement, les vagues tiennent. Vous jouez avec l'élan, ensemble. Le bois est devenu une rive. L'oreiller rayé a fait le tour, sans se taire. Le camp est là, tout bas.</t>
+          <t>On fait des vagues. Tu rebondis, puis tu t'arrêtes. L'oreiller voyage d'un genou à l'autre. Le bois devient une mer, puis une rive. Doucement, les vagues tiennent. Vous avez joué, puis calmé le lit. Le pied du lit est une grotte. L'oreiller rayé a trouvé son coin. Le camp est là, tout bas.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15620,12 +15617,12 @@
         <is>
           <t>enfant-m|On fait des vagues.
 papa|Tu rebondis, puis tu t'arrêtes.
-narrateur|L'oreiller rayé voyage d'un genou à l'autre.
-narrateur|Ils avancent au pied du lit, l'un après l'autre.
+narrateur|L'oreiller voyage d'un genou à l'autre.
+narrateur|Le bois devient une mer, puis une rive.
 enfant-m|Doucement, les vagues tiennent.
-maman|Vous jouez avec l'élan, ensemble.
-papa|Le bois est devenu une rive.
-narrateur|L'oreiller rayé a fait le tour, sans se taire.
+maman|Vous avez joué, puis calmé le lit.
+papa|Le pied du lit est une grotte.
+narrateur|L'oreiller rayé a trouvé son coin.
 enfant-m|Le camp est là, tout bas.</t>
         </is>
       </c>
@@ -15653,12 +15650,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Les vagues s'arrêtent contre le pied du lit. On est arrivés, tous les deux. Tu rebondissais, puis tu t'arrêtais. Le bois est redevenu un lit, simplement. L'élan s'est couché. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière tourne encore, puis tombe. On s'allonge, les vagues se taisent. Dans la chambre, le camp redevient calme.</t>
+          <t>Nino s'allonge au pied du lit. Les vagues sont finies, papa. Tu rebondissais, puis tu t'arrêtais. La grotte a son camp, ce soir. Le bois est redevenu un lit. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière tourne encore, puis tombe. Les vagues se taisent. Dans la chambre, le camp tient.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Les vagues s'arrêtent contre le pied du lit. On est arrivés, tous les deux. Tu rebondissais, puis tu t'arrêtais. Le bois est redevenu un lit, simplement. L'élan s'est couché. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière tourne encore, puis tombe. On s'allonge, les vagues se taisent. Dans la chambre, le camp redevient calme.</t>
+          <t>Nino s'allonge au pied du lit. Les vagues sont finies, papa. Tu rebondissais, puis tu t'arrêtais. La grotte a son camp, ce soir. Le bois est redevenu un lit. L'oreiller rayé garde une chaleur ronde, au creux. Une poussière tourne encore, puis tombe. Les vagues se taisent. Dans la chambre, le camp tient.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15793,15 +15790,15 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|Les vagues s'arrêtent contre le pied du lit.
-enfant-m|On est arrivés, tous les deux.
+          <t>narrateur|Nino s'allonge au pied du lit.
+enfant-m|Les vagues sont finies, papa.
 papa|Tu rebondissais, puis tu t'arrêtais.
-maman|Le bois est redevenu un lit, simplement.
-narrateur|L'élan s'est couché.
+maman|La grotte a son camp, ce soir.
+narrateur|Le bois est redevenu un lit.
 narrateur|L'oreiller rayé garde une chaleur ronde, au creux.
 narrateur|Une poussière tourne encore, puis tombe.
-enfant-m|On s'allonge, les vagues se taisent.
-narrateur|Dans la chambre, le camp redevient calme.</t>
+enfant-m|Les vagues se taisent.
+narrateur|Dans la chambre, le camp tient.</t>
         </is>
       </c>
     </row>
@@ -15828,12 +15825,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. L'oreiller rayé reste muet, au creux. Le matelas se tait, enfin. Maintenant ! Vous avez laissé le bois s'ouvrir. L'élan a attendu le pied. Un pli du drap retombe, tout lent.</t>
+          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. L'oreiller reste sage, au creux du bois. Le matelas se tait, enfin. Maintenant ! Le lit a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. L'oreiller rayé reste muet, au creux. Le matelas se tait, enfin. Maintenant ! Vous avez laissé le bois s'ouvrir. L'élan a attendu le pied. Un pli du drap retombe, tout lent.</t>
+          <t>On attend le matelas. Quand il se tait, tu t'allonges. Un saut, puis le bois reste calme. L'oreiller reste sage, au creux du bois. Le matelas se tait, enfin. Maintenant ! Le lit a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15971,11 +15968,11 @@
           <t>enfant-m|On attend le matelas.
 papa|Quand il se tait, tu t'allonges.
 narrateur|Un saut, puis le bois reste calme.
-narrateur|L'oreiller rayé reste muet, au creux.
+narrateur|L'oreiller reste sage, au creux du bois.
 narrateur|Le matelas se tait, enfin.
 enfant-m|Maintenant !
-maman|Vous avez laissé le bois s'ouvrir.
-papa|L'élan a attendu le pied.
+maman|Le lit a fini ses vagues.
+papa|Tes genoux se sont assis, eux aussi.
 narrateur|Un pli du drap retombe, tout lent.</t>
         </is>
       </c>
@@ -16003,12 +16000,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le matelas s'est tu, enfin, tout à fait. On a attendu le bois. Quand il était calme, on s'allongeait. Le pied vous a laissé le sac. L'élan a écouté le bois. L'oreiller rayé ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
+          <t>Nino s'allonge, le matelas tout calme. On a attendu le bois. Quand il s'est tu, tu es entré. Le pied du lit a fait un toit. Tes genoux se sont assis. L'oreiller rayé ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Le matelas s'est tu, enfin, tout à fait. On a attendu le bois. Quand il était calme, on s'allongeait. Le pied vous a laissé le sac. L'élan a écouté le bois. L'oreiller rayé ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
+          <t>Nino s'allonge, le matelas tout calme. On a attendu le bois. Quand il s'est tu, tu es entré. Le pied du lit a fait un toit. Tes genoux se sont assis. L'oreiller rayé ne fait plus aucun bruit. Nino pose la paume sur le bois tiède. Il est tiède. Un grillon passe derrière le volet, sans crier.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16143,11 +16140,11 @@
       <c r="AV85" s="2" t="inlineStr"/>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>narrateur|Le matelas s'est tu, enfin, tout à fait.
+          <t>narrateur|Nino s'allonge, le matelas tout calme.
 enfant-m|On a attendu le bois.
-papa|Quand il était calme, on s'allongeait.
-maman|Le pied vous a laissé le sac.
-narrateur|L'élan a écouté le bois.
+papa|Quand il s'est tu, tu es entré.
+maman|Le pied du lit a fait un toit.
+narrateur|Tes genoux se sont assis.
 narrateur|L'oreiller rayé ne fait plus aucun bruit.
 narrateur|Nino pose la paume sur le bois tiède.
 enfant-m|Il est tiède.
@@ -16178,12 +16175,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac autour de l'oreiller. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit se range derrière le sac. Vous avez demandé le bord. Mes mains ont tenu l'élan.</t>
+          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac autour de l'oreiller. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit devient un toit. Vous avez demandé le bord. Mes mains ont tenu le camp.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac autour de l'oreiller. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit se range derrière le sac. Vous avez demandé le bord. Mes mains ont tenu l'élan.</t>
+          <t>Maman, tu bordes le sac ? Je le borde, tout chaud. Maman borde le sac autour de l'oreiller. Nino écoute les mains, plus que ses pieds. Tu t'allonges, et ça tient. Moi aussi, j'écoute. Le pied du lit devient un toit. Vous avez demandé le bord. Mes mains ont tenu le camp.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16324,9 +16321,9 @@
 narrateur|Nino écoute les mains, plus que ses pieds.
 papa|Tu t'allonges, et ça tient.
 enfant-m|Moi aussi, j'écoute.
-narrateur|Le pied du lit se range derrière le sac.
+narrateur|Le pied du lit devient un toit.
 papa|Vous avez demandé le bord.
-maman|Mes mains ont tenu l'élan.</t>
+maman|Mes mains ont tenu le camp.</t>
         </is>
       </c>
     </row>
@@ -16353,12 +16350,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Les mains de maman s'éteignent, un à un. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. L'oreiller rayé garde une chaleur ronde, au creux. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
+          <t>Nino s'allonge, le sac bordé par maman. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. L'oreiller rayé garde une chaleur ronde, au creux. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Les mains de maman s'éteignent, un à un. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. L'oreiller rayé garde une chaleur ronde, au creux. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
+          <t>Nino s'allonge, le sac bordé par maman. J'écoutais tes mains. Moi aussi, je bordais avec toi. Vous avez demandé le bord. Le lit a rendu vos pas. L'oreiller rayé garde une chaleur ronde, au creux. Nino touche le sac, du bout des doigts. Il est à nous, maman. Le coton garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16493,7 +16490,7 @@
       <c r="AV87" s="2" t="inlineStr"/>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|Les mains de maman s'éteignent, un à un.
+          <t>narrateur|Nino s'allonge, le sac bordé par maman.
 enfant-m|J'écoutais tes mains.
 papa|Moi aussi, je bordais avec toi.
 maman|Vous avez demandé le bord.
@@ -16522,7 +16519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16565,6 +16562,13 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>